<commit_message>
Fold Templates and Innovate26 into single sections with expandable rows; gradient Excel header
Templates is one section with four rows (PowerPoint, The Brief, Event backdrops, Excel).
Innovate becomes one Innovate26 section with Identity and Applications rows, and the
name loses its space everywhere. Deep links into a row open it and scroll to it on load.
Excel chart templates get a modern gradient header banner.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/site/assets/downloads/SmartCommunications_Excel_Chart_Templates.xlsx
+++ b/site/assets/downloads/SmartCommunications_Excel_Chart_Templates.xlsx
@@ -84,7 +84,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -94,11 +94,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="000E2030"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00326EEF"/>
       </patternFill>
     </fill>
     <fill>
@@ -154,35 +149,34 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="165" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -192,17 +186,17 @@
     <xf numFmtId="9" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="9" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="9" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2392,12 +2386,12 @@
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>22</col>
+      <col>0</col>
       <colOff>0</colOff>
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1123950" cy="371475"/>
+    <ext cx="23936325" cy="609600"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -2422,12 +2416,12 @@
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>22</col>
+      <col>0</col>
       <colOff>0</colOff>
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1123950" cy="371475"/>
+    <ext cx="25946100" cy="609600"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -2474,12 +2468,12 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>22</col>
+      <col>0</col>
       <colOff>0</colOff>
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1123950" cy="371475"/>
+    <ext cx="23660100" cy="609600"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>
@@ -2526,12 +2520,12 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>22</col>
+      <col>0</col>
       <colOff>0</colOff>
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1123950" cy="371475"/>
+    <ext cx="23660100" cy="609600"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>
@@ -2578,12 +2572,12 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>22</col>
+      <col>0</col>
       <colOff>0</colOff>
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1123950" cy="371475"/>
+    <ext cx="23660100" cy="609600"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>
@@ -2630,12 +2624,12 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>22</col>
+      <col>0</col>
       <colOff>0</colOff>
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1123950" cy="371475"/>
+    <ext cx="23660100" cy="609600"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>
@@ -2682,12 +2676,12 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>22</col>
+      <col>0</col>
       <colOff>0</colOff>
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1123950" cy="371475"/>
+    <ext cx="23660100" cy="609600"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>
@@ -2734,12 +2728,12 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>22</col>
+      <col>0</col>
       <colOff>0</colOff>
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1123950" cy="371475"/>
+    <ext cx="24079200" cy="609600"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>
@@ -2786,12 +2780,12 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>22</col>
+      <col>0</col>
       <colOff>0</colOff>
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1123950" cy="371475"/>
+    <ext cx="23660100" cy="609600"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>
@@ -2816,12 +2810,12 @@
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>22</col>
+      <col>0</col>
       <colOff>0</colOff>
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1123950" cy="371475"/>
+    <ext cx="24212550" cy="609600"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -3166,7 +3160,7 @@
     <col width="13" customWidth="1" min="29" max="29"/>
   </cols>
   <sheetData>
-    <row r="1" ht="44" customHeight="1">
+    <row r="1" ht="48" customHeight="1">
       <c r="A1" s="1" t="n"/>
       <c r="B1" s="2" t="inlineStr">
         <is>
@@ -3197,135 +3191,109 @@
       <c r="X1" s="1" t="n"/>
       <c r="Y1" s="1" t="n"/>
     </row>
-    <row r="2" ht="4" customHeight="1">
-      <c r="A2" s="3" t="n"/>
-      <c r="B2" s="3" t="n"/>
-      <c r="C2" s="3" t="n"/>
-      <c r="D2" s="3" t="n"/>
-      <c r="E2" s="3" t="n"/>
-      <c r="F2" s="3" t="n"/>
-      <c r="G2" s="3" t="n"/>
-      <c r="H2" s="3" t="n"/>
-      <c r="I2" s="3" t="n"/>
-      <c r="J2" s="3" t="n"/>
-      <c r="K2" s="3" t="n"/>
-      <c r="L2" s="3" t="n"/>
-      <c r="M2" s="3" t="n"/>
-      <c r="N2" s="3" t="n"/>
-      <c r="O2" s="3" t="n"/>
-      <c r="P2" s="3" t="n"/>
-      <c r="Q2" s="3" t="n"/>
-      <c r="R2" s="3" t="n"/>
-      <c r="S2" s="3" t="n"/>
-      <c r="T2" s="3" t="n"/>
-      <c r="U2" s="3" t="n"/>
-      <c r="V2" s="3" t="n"/>
-      <c r="W2" s="3" t="n"/>
-      <c r="X2" s="3" t="n"/>
-      <c r="Y2" s="3" t="n"/>
-    </row>
+    <row r="2" ht="6" customHeight="1"/>
     <row r="4">
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>How to use</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>1. Pick the tab for the chart you need. Each one has sample data and a finished chart.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>2. Replace the sample data in the light-blue cells (dark blue text). Charts and formulas update automatically.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>3. Edit the chart title in the 'Chart title' cell above the table.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>4. To use a chart in PowerPoint or Word, copy it and paste with 'Keep Source Formatting', or paste as a picture.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="5" t="inlineStr"/>
+      <c r="B9" s="4" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>Cell styles</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>Light-blue cell, dark blue text = edit me · plain cell, navy text = formula or label, leave it</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="5" t="inlineStr"/>
+      <c r="B12" s="4" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="B13" s="4" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>Tabs</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>Column · Column (dark) · Bar · Stacked · Line · Combo · Doughnut · Table · Palette</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="5" t="inlineStr"/>
+      <c r="B15" s="4" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="B16" s="4" t="inlineStr">
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>Brand notes</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="5" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>Type is Segoe UI, the brand's font for Office files. Colors follow the brand chart order (see Palette).</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="B18" s="5" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>The workbook theme is set to the brand colors and font, so Insert → Chart also starts on brand.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="5" t="inlineStr">
+      <c r="B19" s="4" t="inlineStr">
         <is>
           <t>All sample numbers are illustrative.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="6" t="inlineStr">
+      <c r="B21" s="5" t="inlineStr">
         <is>
           <t>Example input cell</t>
         </is>
@@ -3380,7 +3348,7 @@
     <col width="13" customWidth="1" min="29" max="29"/>
   </cols>
   <sheetData>
-    <row r="1" ht="44" customHeight="1">
+    <row r="1" ht="48" customHeight="1">
       <c r="A1" s="1" t="n"/>
       <c r="B1" s="2" t="inlineStr">
         <is>
@@ -3411,265 +3379,239 @@
       <c r="X1" s="1" t="n"/>
       <c r="Y1" s="1" t="n"/>
     </row>
-    <row r="2" ht="4" customHeight="1">
-      <c r="A2" s="3" t="n"/>
-      <c r="B2" s="3" t="n"/>
-      <c r="C2" s="3" t="n"/>
-      <c r="D2" s="3" t="n"/>
-      <c r="E2" s="3" t="n"/>
-      <c r="F2" s="3" t="n"/>
-      <c r="G2" s="3" t="n"/>
-      <c r="H2" s="3" t="n"/>
-      <c r="I2" s="3" t="n"/>
-      <c r="J2" s="3" t="n"/>
-      <c r="K2" s="3" t="n"/>
-      <c r="L2" s="3" t="n"/>
-      <c r="M2" s="3" t="n"/>
-      <c r="N2" s="3" t="n"/>
-      <c r="O2" s="3" t="n"/>
-      <c r="P2" s="3" t="n"/>
-      <c r="Q2" s="3" t="n"/>
-      <c r="R2" s="3" t="n"/>
-      <c r="S2" s="3" t="n"/>
-      <c r="T2" s="3" t="n"/>
-      <c r="U2" s="3" t="n"/>
-      <c r="V2" s="3" t="n"/>
-      <c r="W2" s="3" t="n"/>
-      <c r="X2" s="3" t="n"/>
-      <c r="Y2" s="3" t="n"/>
-    </row>
+    <row r="2" ht="6" customHeight="1"/>
     <row r="4">
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Use the colors in this order. The workbook theme carries the same order, so new charts start on brand.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="20" t="inlineStr">
+      <c r="B7" s="19" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="C7" s="20" t="inlineStr">
+      <c r="C7" s="19" t="inlineStr">
         <is>
           <t>Color</t>
         </is>
       </c>
-      <c r="D7" s="20" t="inlineStr">
+      <c r="D7" s="19" t="inlineStr">
         <is>
           <t>HEX</t>
         </is>
       </c>
-      <c r="E7" s="20" t="inlineStr">
+      <c r="E7" s="19" t="inlineStr">
         <is>
           <t>Swatch</t>
         </is>
       </c>
-      <c r="F7" s="20" t="inlineStr">
+      <c r="F7" s="19" t="inlineStr">
         <is>
           <t>Use for</t>
         </is>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="B8" s="21" t="inlineStr">
+      <c r="B8" s="20" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="C8" s="21" t="inlineStr">
+      <c r="C8" s="20" t="inlineStr">
         <is>
           <t>Dodger</t>
         </is>
       </c>
-      <c r="D8" s="21" t="inlineStr">
+      <c r="D8" s="20" t="inlineStr">
         <is>
           <t>#0094FF</t>
         </is>
       </c>
-      <c r="E8" s="22" t="inlineStr"/>
-      <c r="F8" s="21" t="inlineStr">
+      <c r="E8" s="21" t="inlineStr"/>
+      <c r="F8" s="20" t="inlineStr">
         <is>
           <t>Lead series. Single-series charts use only this</t>
         </is>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="B9" s="21" t="inlineStr">
+      <c r="B9" s="20" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="C9" s="21" t="inlineStr">
+      <c r="C9" s="20" t="inlineStr">
         <is>
           <t>Indigo Dark</t>
         </is>
       </c>
-      <c r="D9" s="21" t="inlineStr">
+      <c r="D9" s="20" t="inlineStr">
         <is>
           <t>#661DEE</t>
         </is>
       </c>
-      <c r="E9" s="23" t="inlineStr"/>
-      <c r="F9" s="21" t="inlineStr">
+      <c r="E9" s="22" t="inlineStr"/>
+      <c r="F9" s="20" t="inlineStr">
         <is>
           <t>Second series, targets and comparisons</t>
         </is>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="B10" s="21" t="inlineStr">
+      <c r="B10" s="20" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="C10" s="21" t="inlineStr">
+      <c r="C10" s="20" t="inlineStr">
         <is>
           <t>Dodger Light</t>
         </is>
       </c>
-      <c r="D10" s="21" t="inlineStr">
+      <c r="D10" s="20" t="inlineStr">
         <is>
           <t>#57B8FF</t>
         </is>
       </c>
-      <c r="E10" s="24" t="inlineStr"/>
-      <c r="F10" s="21" t="inlineStr">
+      <c r="E10" s="23" t="inlineStr"/>
+      <c r="F10" s="20" t="inlineStr">
         <is>
           <t>Third series</t>
         </is>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="B11" s="21" t="inlineStr">
+      <c r="B11" s="20" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="C11" s="21" t="inlineStr">
+      <c r="C11" s="20" t="inlineStr">
         <is>
           <t>UI Blue Dark</t>
         </is>
       </c>
-      <c r="D11" s="21" t="inlineStr">
+      <c r="D11" s="20" t="inlineStr">
         <is>
           <t>#1344C1</t>
         </is>
       </c>
-      <c r="E11" s="25" t="inlineStr"/>
-      <c r="F11" s="21" t="inlineStr">
+      <c r="E11" s="24" t="inlineStr"/>
+      <c r="F11" s="20" t="inlineStr">
         <is>
           <t>Fourth series</t>
         </is>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="B12" s="21" t="inlineStr">
+      <c r="B12" s="20" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="C12" s="21" t="inlineStr">
+      <c r="C12" s="20" t="inlineStr">
         <is>
           <t>Indigo Light</t>
         </is>
       </c>
-      <c r="D12" s="21" t="inlineStr">
+      <c r="D12" s="20" t="inlineStr">
         <is>
           <t>#BE9DFA</t>
         </is>
       </c>
-      <c r="E12" s="26" t="inlineStr"/>
-      <c r="F12" s="21" t="inlineStr">
+      <c r="E12" s="25" t="inlineStr"/>
+      <c r="F12" s="20" t="inlineStr">
         <is>
           <t>Fifth series</t>
         </is>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="B13" s="21" t="inlineStr">
+      <c r="B13" s="20" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="C13" s="21" t="inlineStr">
+      <c r="C13" s="20" t="inlineStr">
         <is>
           <t>Dodger Dark</t>
         </is>
       </c>
-      <c r="D13" s="21" t="inlineStr">
+      <c r="D13" s="20" t="inlineStr">
         <is>
           <t>#0062A8</t>
         </is>
       </c>
-      <c r="E13" s="27" t="inlineStr"/>
-      <c r="F13" s="21" t="inlineStr">
+      <c r="E13" s="26" t="inlineStr"/>
+      <c r="F13" s="20" t="inlineStr">
         <is>
           <t>Sixth series, or fold the rest into 'Other'</t>
         </is>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="B14" s="21" t="inlineStr">
+      <c r="B14" s="20" t="inlineStr">
         <is>
           <t>Dark</t>
         </is>
       </c>
-      <c r="C14" s="21" t="inlineStr">
+      <c r="C14" s="20" t="inlineStr">
         <is>
           <t>On Tiber slides</t>
         </is>
       </c>
-      <c r="D14" s="21" t="inlineStr">
+      <c r="D14" s="20" t="inlineStr">
         <is>
           <t>#0094FF · #661DEE · #0062A8 · #9963FD</t>
         </is>
       </c>
-      <c r="E14" s="21" t="inlineStr"/>
-      <c r="F14" s="21" t="inlineStr">
+      <c r="E14" s="20" t="inlineStr"/>
+      <c r="F14" s="20" t="inlineStr">
         <is>
           <t>Four series at most on dark</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>•  Keep it to five or six series; past that, group the smallest into 'Other'.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>•  One series? Use Dodger alone. More? Follow the order above so neighbors stay easy to tell apart.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="5" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>•  No rainbow or traffic-light colors. Show status with labels or shades of blue.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="B18" s="5" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>•  Text in charts is Segoe UI. On dark (Tiber) slides use the 'Column (dark)' style and the dark order.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="5" t="inlineStr">
+      <c r="B19" s="4" t="inlineStr">
         <is>
           <t>•  The order is checked for colorblind readers too; keep the data table or labels with lighter colors.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="5" t="inlineStr">
+      <c r="B20" s="4" t="inlineStr">
         <is>
           <t>•  Label illustrative numbers as illustrative, and cite real data under the table.</t>
         </is>
@@ -3724,7 +3666,7 @@
     <col width="13" customWidth="1" min="29" max="29"/>
   </cols>
   <sheetData>
-    <row r="1" ht="44" customHeight="1">
+    <row r="1" ht="48" customHeight="1">
       <c r="A1" s="1" t="n"/>
       <c r="B1" s="2" t="inlineStr">
         <is>
@@ -3755,176 +3697,150 @@
       <c r="X1" s="1" t="n"/>
       <c r="Y1" s="1" t="n"/>
     </row>
-    <row r="2" ht="4" customHeight="1">
-      <c r="A2" s="3" t="n"/>
-      <c r="B2" s="3" t="n"/>
-      <c r="C2" s="3" t="n"/>
-      <c r="D2" s="3" t="n"/>
-      <c r="E2" s="3" t="n"/>
-      <c r="F2" s="3" t="n"/>
-      <c r="G2" s="3" t="n"/>
-      <c r="H2" s="3" t="n"/>
-      <c r="I2" s="3" t="n"/>
-      <c r="J2" s="3" t="n"/>
-      <c r="K2" s="3" t="n"/>
-      <c r="L2" s="3" t="n"/>
-      <c r="M2" s="3" t="n"/>
-      <c r="N2" s="3" t="n"/>
-      <c r="O2" s="3" t="n"/>
-      <c r="P2" s="3" t="n"/>
-      <c r="Q2" s="3" t="n"/>
-      <c r="R2" s="3" t="n"/>
-      <c r="S2" s="3" t="n"/>
-      <c r="T2" s="3" t="n"/>
-      <c r="U2" s="3" t="n"/>
-      <c r="V2" s="3" t="n"/>
-      <c r="W2" s="3" t="n"/>
-      <c r="X2" s="3" t="n"/>
-      <c r="Y2" s="3" t="n"/>
-    </row>
+    <row r="2" ht="6" customHeight="1"/>
     <row r="4">
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Edit the light-blue cells: the chart updates automatically. Copy the chart into PowerPoint or Word.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>Chart title</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>Communications sent by channel</t>
         </is>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>Quarter</t>
         </is>
       </c>
-      <c r="C9" s="10" t="inlineStr">
+      <c r="C9" s="9" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="D9" s="10" t="inlineStr">
+      <c r="D9" s="9" t="inlineStr">
         <is>
           <t>Print</t>
         </is>
       </c>
-      <c r="E9" s="10" t="inlineStr">
+      <c r="E9" s="9" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="F9" s="10" t="inlineStr">
+      <c r="F9" s="9" t="inlineStr">
         <is>
           <t>Portal</t>
         </is>
       </c>
-      <c r="G9" s="10" t="inlineStr">
+      <c r="G9" s="9" t="inlineStr">
         <is>
           <t>App</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="11" t="inlineStr">
+      <c r="B10" s="10" t="inlineStr">
         <is>
           <t>Q1</t>
         </is>
       </c>
-      <c r="C10" s="12" t="n">
+      <c r="C10" s="11" t="n">
         <v>42000</v>
       </c>
-      <c r="D10" s="12" t="n">
+      <c r="D10" s="11" t="n">
         <v>31000</v>
       </c>
-      <c r="E10" s="12" t="n">
+      <c r="E10" s="11" t="n">
         <v>12000</v>
       </c>
-      <c r="F10" s="12" t="n">
+      <c r="F10" s="11" t="n">
         <v>21000</v>
       </c>
-      <c r="G10" s="12" t="n">
+      <c r="G10" s="11" t="n">
         <v>8000</v>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="11" t="inlineStr">
+      <c r="B11" s="10" t="inlineStr">
         <is>
           <t>Q2</t>
         </is>
       </c>
-      <c r="C11" s="12" t="n">
+      <c r="C11" s="11" t="n">
         <v>46500</v>
       </c>
-      <c r="D11" s="12" t="n">
+      <c r="D11" s="11" t="n">
         <v>29800</v>
       </c>
-      <c r="E11" s="12" t="n">
+      <c r="E11" s="11" t="n">
         <v>15400</v>
       </c>
-      <c r="F11" s="12" t="n">
+      <c r="F11" s="11" t="n">
         <v>24000</v>
       </c>
-      <c r="G11" s="12" t="n">
+      <c r="G11" s="11" t="n">
         <v>11500</v>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="11" t="inlineStr">
+      <c r="B12" s="10" t="inlineStr">
         <is>
           <t>Q3</t>
         </is>
       </c>
-      <c r="C12" s="12" t="n">
+      <c r="C12" s="11" t="n">
         <v>51200</v>
       </c>
-      <c r="D12" s="12" t="n">
+      <c r="D12" s="11" t="n">
         <v>27600</v>
       </c>
-      <c r="E12" s="12" t="n">
+      <c r="E12" s="11" t="n">
         <v>18900</v>
       </c>
-      <c r="F12" s="12" t="n">
+      <c r="F12" s="11" t="n">
         <v>26500</v>
       </c>
-      <c r="G12" s="12" t="n">
+      <c r="G12" s="11" t="n">
         <v>15800</v>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="11" t="inlineStr">
+      <c r="B13" s="10" t="inlineStr">
         <is>
           <t>Q4</t>
         </is>
       </c>
-      <c r="C13" s="12" t="n">
+      <c r="C13" s="11" t="n">
         <v>55800</v>
       </c>
-      <c r="D13" s="12" t="n">
+      <c r="D13" s="11" t="n">
         <v>26100</v>
       </c>
-      <c r="E13" s="12" t="n">
+      <c r="E13" s="11" t="n">
         <v>22300</v>
       </c>
-      <c r="F13" s="12" t="n">
+      <c r="F13" s="11" t="n">
         <v>29900</v>
       </c>
-      <c r="G13" s="12" t="n">
+      <c r="G13" s="11" t="n">
         <v>19400</v>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="7" t="inlineStr">
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>Sample data is illustrative. Replace it with your own and cite the source under the table.</t>
         </is>
@@ -3982,7 +3898,7 @@
     <col width="13" customWidth="1" min="29" max="29"/>
   </cols>
   <sheetData>
-    <row r="1" ht="44" customHeight="1">
+    <row r="1" ht="48" customHeight="1">
       <c r="A1" s="1" t="n"/>
       <c r="B1" s="2" t="inlineStr">
         <is>
@@ -4013,159 +3929,133 @@
       <c r="X1" s="1" t="n"/>
       <c r="Y1" s="1" t="n"/>
     </row>
-    <row r="2" ht="4" customHeight="1">
-      <c r="A2" s="3" t="n"/>
-      <c r="B2" s="3" t="n"/>
-      <c r="C2" s="3" t="n"/>
-      <c r="D2" s="3" t="n"/>
-      <c r="E2" s="3" t="n"/>
-      <c r="F2" s="3" t="n"/>
-      <c r="G2" s="3" t="n"/>
-      <c r="H2" s="3" t="n"/>
-      <c r="I2" s="3" t="n"/>
-      <c r="J2" s="3" t="n"/>
-      <c r="K2" s="3" t="n"/>
-      <c r="L2" s="3" t="n"/>
-      <c r="M2" s="3" t="n"/>
-      <c r="N2" s="3" t="n"/>
-      <c r="O2" s="3" t="n"/>
-      <c r="P2" s="3" t="n"/>
-      <c r="Q2" s="3" t="n"/>
-      <c r="R2" s="3" t="n"/>
-      <c r="S2" s="3" t="n"/>
-      <c r="T2" s="3" t="n"/>
-      <c r="U2" s="3" t="n"/>
-      <c r="V2" s="3" t="n"/>
-      <c r="W2" s="3" t="n"/>
-      <c r="X2" s="3" t="n"/>
-      <c r="Y2" s="3" t="n"/>
-    </row>
+    <row r="2" ht="6" customHeight="1"/>
     <row r="4">
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Edit the light-blue cells: the chart updates automatically. Copy the chart into PowerPoint or Word. This version is styled for Tiber (dark) slides.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>Chart title</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>Communications sent by channel</t>
         </is>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>Quarter</t>
         </is>
       </c>
-      <c r="C9" s="10" t="inlineStr">
+      <c r="C9" s="9" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="D9" s="10" t="inlineStr">
+      <c r="D9" s="9" t="inlineStr">
         <is>
           <t>Print</t>
         </is>
       </c>
-      <c r="E9" s="10" t="inlineStr">
+      <c r="E9" s="9" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="F9" s="10" t="inlineStr">
+      <c r="F9" s="9" t="inlineStr">
         <is>
           <t>Portal</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="11" t="inlineStr">
+      <c r="B10" s="10" t="inlineStr">
         <is>
           <t>Q1</t>
         </is>
       </c>
-      <c r="C10" s="12" t="n">
+      <c r="C10" s="11" t="n">
         <v>42000</v>
       </c>
-      <c r="D10" s="12" t="n">
+      <c r="D10" s="11" t="n">
         <v>31000</v>
       </c>
-      <c r="E10" s="12" t="n">
+      <c r="E10" s="11" t="n">
         <v>12000</v>
       </c>
-      <c r="F10" s="12" t="n">
+      <c r="F10" s="11" t="n">
         <v>21000</v>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="11" t="inlineStr">
+      <c r="B11" s="10" t="inlineStr">
         <is>
           <t>Q2</t>
         </is>
       </c>
-      <c r="C11" s="12" t="n">
+      <c r="C11" s="11" t="n">
         <v>46500</v>
       </c>
-      <c r="D11" s="12" t="n">
+      <c r="D11" s="11" t="n">
         <v>29800</v>
       </c>
-      <c r="E11" s="12" t="n">
+      <c r="E11" s="11" t="n">
         <v>15400</v>
       </c>
-      <c r="F11" s="12" t="n">
+      <c r="F11" s="11" t="n">
         <v>24000</v>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="11" t="inlineStr">
+      <c r="B12" s="10" t="inlineStr">
         <is>
           <t>Q3</t>
         </is>
       </c>
-      <c r="C12" s="12" t="n">
+      <c r="C12" s="11" t="n">
         <v>51200</v>
       </c>
-      <c r="D12" s="12" t="n">
+      <c r="D12" s="11" t="n">
         <v>27600</v>
       </c>
-      <c r="E12" s="12" t="n">
+      <c r="E12" s="11" t="n">
         <v>18900</v>
       </c>
-      <c r="F12" s="12" t="n">
+      <c r="F12" s="11" t="n">
         <v>26500</v>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="11" t="inlineStr">
+      <c r="B13" s="10" t="inlineStr">
         <is>
           <t>Q4</t>
         </is>
       </c>
-      <c r="C13" s="12" t="n">
+      <c r="C13" s="11" t="n">
         <v>55800</v>
       </c>
-      <c r="D13" s="12" t="n">
+      <c r="D13" s="11" t="n">
         <v>26100</v>
       </c>
-      <c r="E13" s="12" t="n">
+      <c r="E13" s="11" t="n">
         <v>22300</v>
       </c>
-      <c r="F13" s="12" t="n">
+      <c r="F13" s="11" t="n">
         <v>29900</v>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="7" t="inlineStr">
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>Sample data is illustrative. Replace it with your own and cite the source under the table.</t>
         </is>
@@ -4223,7 +4113,7 @@
     <col width="13" customWidth="1" min="29" max="29"/>
   </cols>
   <sheetData>
-    <row r="1" ht="44" customHeight="1">
+    <row r="1" ht="48" customHeight="1">
       <c r="A1" s="1" t="n"/>
       <c r="B1" s="2" t="inlineStr">
         <is>
@@ -4254,128 +4144,102 @@
       <c r="X1" s="1" t="n"/>
       <c r="Y1" s="1" t="n"/>
     </row>
-    <row r="2" ht="4" customHeight="1">
-      <c r="A2" s="3" t="n"/>
-      <c r="B2" s="3" t="n"/>
-      <c r="C2" s="3" t="n"/>
-      <c r="D2" s="3" t="n"/>
-      <c r="E2" s="3" t="n"/>
-      <c r="F2" s="3" t="n"/>
-      <c r="G2" s="3" t="n"/>
-      <c r="H2" s="3" t="n"/>
-      <c r="I2" s="3" t="n"/>
-      <c r="J2" s="3" t="n"/>
-      <c r="K2" s="3" t="n"/>
-      <c r="L2" s="3" t="n"/>
-      <c r="M2" s="3" t="n"/>
-      <c r="N2" s="3" t="n"/>
-      <c r="O2" s="3" t="n"/>
-      <c r="P2" s="3" t="n"/>
-      <c r="Q2" s="3" t="n"/>
-      <c r="R2" s="3" t="n"/>
-      <c r="S2" s="3" t="n"/>
-      <c r="T2" s="3" t="n"/>
-      <c r="U2" s="3" t="n"/>
-      <c r="V2" s="3" t="n"/>
-      <c r="W2" s="3" t="n"/>
-      <c r="X2" s="3" t="n"/>
-      <c r="Y2" s="3" t="n"/>
-    </row>
+    <row r="2" ht="6" customHeight="1"/>
     <row r="4">
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Horizontal bars for ranked lists. Sort the table from largest to smallest; the chart keeps the same order.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>Chart title</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>Templates migrated by business unit</t>
         </is>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>Business unit</t>
         </is>
       </c>
-      <c r="C9" s="10" t="inlineStr">
+      <c r="C9" s="9" t="inlineStr">
         <is>
           <t>Templates</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="11" t="inlineStr">
+      <c r="B10" s="10" t="inlineStr">
         <is>
           <t>Claims</t>
         </is>
       </c>
-      <c r="C10" s="12" t="n">
+      <c r="C10" s="11" t="n">
         <v>412</v>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="11" t="inlineStr">
+      <c r="B11" s="10" t="inlineStr">
         <is>
           <t>Policy servicing</t>
         </is>
       </c>
-      <c r="C11" s="12" t="n">
+      <c r="C11" s="11" t="n">
         <v>356</v>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="11" t="inlineStr">
+      <c r="B12" s="10" t="inlineStr">
         <is>
           <t>Billing</t>
         </is>
       </c>
-      <c r="C12" s="12" t="n">
+      <c r="C12" s="11" t="n">
         <v>298</v>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="11" t="inlineStr">
+      <c r="B13" s="10" t="inlineStr">
         <is>
           <t>Onboarding</t>
         </is>
       </c>
-      <c r="C13" s="12" t="n">
+      <c r="C13" s="11" t="n">
         <v>241</v>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="11" t="inlineStr">
+      <c r="B14" s="10" t="inlineStr">
         <is>
           <t>Complaints</t>
         </is>
       </c>
-      <c r="C14" s="12" t="n">
+      <c r="C14" s="11" t="n">
         <v>167</v>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="11" t="inlineStr">
+      <c r="B15" s="10" t="inlineStr">
         <is>
           <t>Marketing</t>
         </is>
       </c>
-      <c r="C15" s="12" t="n">
+      <c r="C15" s="11" t="n">
         <v>102</v>
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="7" t="inlineStr">
+      <c r="B16" s="6" t="inlineStr">
         <is>
           <t>Sample data is illustrative. Replace it with your own and cite the source under the table.</t>
         </is>
@@ -4433,7 +4297,7 @@
     <col width="13" customWidth="1" min="29" max="29"/>
   </cols>
   <sheetData>
-    <row r="1" ht="44" customHeight="1">
+    <row r="1" ht="48" customHeight="1">
       <c r="A1" s="1" t="n"/>
       <c r="B1" s="2" t="inlineStr">
         <is>
@@ -4464,159 +4328,133 @@
       <c r="X1" s="1" t="n"/>
       <c r="Y1" s="1" t="n"/>
     </row>
-    <row r="2" ht="4" customHeight="1">
-      <c r="A2" s="3" t="n"/>
-      <c r="B2" s="3" t="n"/>
-      <c r="C2" s="3" t="n"/>
-      <c r="D2" s="3" t="n"/>
-      <c r="E2" s="3" t="n"/>
-      <c r="F2" s="3" t="n"/>
-      <c r="G2" s="3" t="n"/>
-      <c r="H2" s="3" t="n"/>
-      <c r="I2" s="3" t="n"/>
-      <c r="J2" s="3" t="n"/>
-      <c r="K2" s="3" t="n"/>
-      <c r="L2" s="3" t="n"/>
-      <c r="M2" s="3" t="n"/>
-      <c r="N2" s="3" t="n"/>
-      <c r="O2" s="3" t="n"/>
-      <c r="P2" s="3" t="n"/>
-      <c r="Q2" s="3" t="n"/>
-      <c r="R2" s="3" t="n"/>
-      <c r="S2" s="3" t="n"/>
-      <c r="T2" s="3" t="n"/>
-      <c r="U2" s="3" t="n"/>
-      <c r="V2" s="3" t="n"/>
-      <c r="W2" s="3" t="n"/>
-      <c r="X2" s="3" t="n"/>
-      <c r="Y2" s="3" t="n"/>
-    </row>
+    <row r="2" ht="6" customHeight="1"/>
     <row r="4">
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Shows how a total splits by channel. Use four series or fewer so the blues stay easy to tell apart.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>Chart title</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>Channel mix by quarter</t>
         </is>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>Quarter</t>
         </is>
       </c>
-      <c r="C9" s="10" t="inlineStr">
+      <c r="C9" s="9" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="D9" s="10" t="inlineStr">
+      <c r="D9" s="9" t="inlineStr">
         <is>
           <t>Portal</t>
         </is>
       </c>
-      <c r="E9" s="10" t="inlineStr">
+      <c r="E9" s="9" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="F9" s="10" t="inlineStr">
+      <c r="F9" s="9" t="inlineStr">
         <is>
           <t>Print</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="11" t="inlineStr">
+      <c r="B10" s="10" t="inlineStr">
         <is>
           <t>Q1</t>
         </is>
       </c>
-      <c r="C10" s="13" t="n">
+      <c r="C10" s="12" t="n">
         <v>38</v>
       </c>
-      <c r="D10" s="13" t="n">
+      <c r="D10" s="12" t="n">
         <v>14</v>
       </c>
-      <c r="E10" s="13" t="n">
+      <c r="E10" s="12" t="n">
         <v>11</v>
       </c>
-      <c r="F10" s="13" t="n">
+      <c r="F10" s="12" t="n">
         <v>37</v>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="11" t="inlineStr">
+      <c r="B11" s="10" t="inlineStr">
         <is>
           <t>Q2</t>
         </is>
       </c>
-      <c r="C11" s="13" t="n">
+      <c r="C11" s="12" t="n">
         <v>41</v>
       </c>
-      <c r="D11" s="13" t="n">
+      <c r="D11" s="12" t="n">
         <v>17</v>
       </c>
-      <c r="E11" s="13" t="n">
+      <c r="E11" s="12" t="n">
         <v>13</v>
       </c>
-      <c r="F11" s="13" t="n">
+      <c r="F11" s="12" t="n">
         <v>29</v>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="11" t="inlineStr">
+      <c r="B12" s="10" t="inlineStr">
         <is>
           <t>Q3</t>
         </is>
       </c>
-      <c r="C12" s="13" t="n">
+      <c r="C12" s="12" t="n">
         <v>44</v>
       </c>
-      <c r="D12" s="13" t="n">
+      <c r="D12" s="12" t="n">
         <v>19</v>
       </c>
-      <c r="E12" s="13" t="n">
+      <c r="E12" s="12" t="n">
         <v>14</v>
       </c>
-      <c r="F12" s="13" t="n">
+      <c r="F12" s="12" t="n">
         <v>23</v>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="11" t="inlineStr">
+      <c r="B13" s="10" t="inlineStr">
         <is>
           <t>Q4</t>
         </is>
       </c>
-      <c r="C13" s="13" t="n">
+      <c r="C13" s="12" t="n">
         <v>46</v>
       </c>
-      <c r="D13" s="13" t="n">
+      <c r="D13" s="12" t="n">
         <v>22</v>
       </c>
-      <c r="E13" s="13" t="n">
+      <c r="E13" s="12" t="n">
         <v>16</v>
       </c>
-      <c r="F13" s="13" t="n">
+      <c r="F13" s="12" t="n">
         <v>16</v>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="7" t="inlineStr">
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>Sample data is illustrative. Replace it with your own and cite the source under the table. Values are percent of volume and add up to 100.</t>
         </is>
@@ -4674,7 +4512,7 @@
     <col width="13" customWidth="1" min="29" max="29"/>
   </cols>
   <sheetData>
-    <row r="1" ht="44" customHeight="1">
+    <row r="1" ht="48" customHeight="1">
       <c r="A1" s="1" t="n"/>
       <c r="B1" s="2" t="inlineStr">
         <is>
@@ -4705,229 +4543,203 @@
       <c r="X1" s="1" t="n"/>
       <c r="Y1" s="1" t="n"/>
     </row>
-    <row r="2" ht="4" customHeight="1">
-      <c r="A2" s="3" t="n"/>
-      <c r="B2" s="3" t="n"/>
-      <c r="C2" s="3" t="n"/>
-      <c r="D2" s="3" t="n"/>
-      <c r="E2" s="3" t="n"/>
-      <c r="F2" s="3" t="n"/>
-      <c r="G2" s="3" t="n"/>
-      <c r="H2" s="3" t="n"/>
-      <c r="I2" s="3" t="n"/>
-      <c r="J2" s="3" t="n"/>
-      <c r="K2" s="3" t="n"/>
-      <c r="L2" s="3" t="n"/>
-      <c r="M2" s="3" t="n"/>
-      <c r="N2" s="3" t="n"/>
-      <c r="O2" s="3" t="n"/>
-      <c r="P2" s="3" t="n"/>
-      <c r="Q2" s="3" t="n"/>
-      <c r="R2" s="3" t="n"/>
-      <c r="S2" s="3" t="n"/>
-      <c r="T2" s="3" t="n"/>
-      <c r="U2" s="3" t="n"/>
-      <c r="V2" s="3" t="n"/>
-      <c r="W2" s="3" t="n"/>
-      <c r="X2" s="3" t="n"/>
-      <c r="Y2" s="3" t="n"/>
-    </row>
+    <row r="2" ht="6" customHeight="1"/>
     <row r="4">
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Monthly trends. Put the current period first so it takes the brand's lead color.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>Chart title</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>Average days to update a template</t>
         </is>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="C9" s="10" t="inlineStr">
+      <c r="C9" s="9" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="D9" s="10" t="inlineStr">
+      <c r="D9" s="9" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="11" t="inlineStr">
+      <c r="B10" s="10" t="inlineStr">
         <is>
           <t>Jan</t>
         </is>
       </c>
-      <c r="C10" s="12" t="n">
+      <c r="C10" s="11" t="n">
         <v>21</v>
       </c>
-      <c r="D10" s="12" t="n">
+      <c r="D10" s="11" t="n">
         <v>24</v>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="11" t="inlineStr">
+      <c r="B11" s="10" t="inlineStr">
         <is>
           <t>Feb</t>
         </is>
       </c>
-      <c r="C11" s="12" t="n">
+      <c r="C11" s="11" t="n">
         <v>19</v>
       </c>
-      <c r="D11" s="12" t="n">
+      <c r="D11" s="11" t="n">
         <v>24</v>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="11" t="inlineStr">
+      <c r="B12" s="10" t="inlineStr">
         <is>
           <t>Mar</t>
         </is>
       </c>
-      <c r="C12" s="12" t="n">
+      <c r="C12" s="11" t="n">
         <v>18</v>
       </c>
-      <c r="D12" s="12" t="n">
+      <c r="D12" s="11" t="n">
         <v>23</v>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="11" t="inlineStr">
+      <c r="B13" s="10" t="inlineStr">
         <is>
           <t>Apr</t>
         </is>
       </c>
-      <c r="C13" s="12" t="n">
+      <c r="C13" s="11" t="n">
         <v>16</v>
       </c>
-      <c r="D13" s="12" t="n">
+      <c r="D13" s="11" t="n">
         <v>23</v>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="11" t="inlineStr">
+      <c r="B14" s="10" t="inlineStr">
         <is>
           <t>May</t>
         </is>
       </c>
-      <c r="C14" s="12" t="n">
+      <c r="C14" s="11" t="n">
         <v>15</v>
       </c>
-      <c r="D14" s="12" t="n">
+      <c r="D14" s="11" t="n">
         <v>22</v>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="11" t="inlineStr">
+      <c r="B15" s="10" t="inlineStr">
         <is>
           <t>Jun</t>
         </is>
       </c>
-      <c r="C15" s="12" t="n">
+      <c r="C15" s="11" t="n">
         <v>13</v>
       </c>
-      <c r="D15" s="12" t="n">
+      <c r="D15" s="11" t="n">
         <v>22</v>
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="11" t="inlineStr">
+      <c r="B16" s="10" t="inlineStr">
         <is>
           <t>Jul</t>
         </is>
       </c>
-      <c r="C16" s="12" t="n">
+      <c r="C16" s="11" t="n">
         <v>12</v>
       </c>
-      <c r="D16" s="12" t="n">
+      <c r="D16" s="11" t="n">
         <v>21</v>
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="11" t="inlineStr">
+      <c r="B17" s="10" t="inlineStr">
         <is>
           <t>Aug</t>
         </is>
       </c>
-      <c r="C17" s="12" t="n">
+      <c r="C17" s="11" t="n">
         <v>11</v>
       </c>
-      <c r="D17" s="12" t="n">
+      <c r="D17" s="11" t="n">
         <v>21</v>
       </c>
     </row>
     <row r="18">
-      <c r="B18" s="11" t="inlineStr">
+      <c r="B18" s="10" t="inlineStr">
         <is>
           <t>Sep</t>
         </is>
       </c>
-      <c r="C18" s="12" t="n">
+      <c r="C18" s="11" t="n">
         <v>10</v>
       </c>
-      <c r="D18" s="12" t="n">
+      <c r="D18" s="11" t="n">
         <v>21</v>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="11" t="inlineStr">
+      <c r="B19" s="10" t="inlineStr">
         <is>
           <t>Oct</t>
         </is>
       </c>
-      <c r="C19" s="12" t="n">
+      <c r="C19" s="11" t="n">
         <v>9</v>
       </c>
-      <c r="D19" s="12" t="n">
+      <c r="D19" s="11" t="n">
         <v>20</v>
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="11" t="inlineStr">
+      <c r="B20" s="10" t="inlineStr">
         <is>
           <t>Nov</t>
         </is>
       </c>
-      <c r="C20" s="12" t="n">
+      <c r="C20" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="D20" s="12" t="n">
+      <c r="D20" s="11" t="n">
         <v>20</v>
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="11" t="inlineStr">
+      <c r="B21" s="10" t="inlineStr">
         <is>
           <t>Dec</t>
         </is>
       </c>
-      <c r="C21" s="12" t="n">
+      <c r="C21" s="11" t="n">
         <v>7</v>
       </c>
-      <c r="D21" s="12" t="n">
+      <c r="D21" s="11" t="n">
         <v>20</v>
       </c>
     </row>
     <row r="22">
-      <c r="B22" s="7" t="inlineStr">
+      <c r="B22" s="6" t="inlineStr">
         <is>
           <t>Sample data is illustrative. Replace it with your own and cite the source under the table.</t>
         </is>
@@ -4985,7 +4797,7 @@
     <col width="13" customWidth="1" min="29" max="29"/>
   </cols>
   <sheetData>
-    <row r="1" ht="44" customHeight="1">
+    <row r="1" ht="48" customHeight="1">
       <c r="A1" s="1" t="n"/>
       <c r="B1" s="2" t="inlineStr">
         <is>
@@ -5016,180 +4828,154 @@
       <c r="X1" s="1" t="n"/>
       <c r="Y1" s="1" t="n"/>
     </row>
-    <row r="2" ht="4" customHeight="1">
-      <c r="A2" s="3" t="n"/>
-      <c r="B2" s="3" t="n"/>
-      <c r="C2" s="3" t="n"/>
-      <c r="D2" s="3" t="n"/>
-      <c r="E2" s="3" t="n"/>
-      <c r="F2" s="3" t="n"/>
-      <c r="G2" s="3" t="n"/>
-      <c r="H2" s="3" t="n"/>
-      <c r="I2" s="3" t="n"/>
-      <c r="J2" s="3" t="n"/>
-      <c r="K2" s="3" t="n"/>
-      <c r="L2" s="3" t="n"/>
-      <c r="M2" s="3" t="n"/>
-      <c r="N2" s="3" t="n"/>
-      <c r="O2" s="3" t="n"/>
-      <c r="P2" s="3" t="n"/>
-      <c r="Q2" s="3" t="n"/>
-      <c r="R2" s="3" t="n"/>
-      <c r="S2" s="3" t="n"/>
-      <c r="T2" s="3" t="n"/>
-      <c r="U2" s="3" t="n"/>
-      <c r="V2" s="3" t="n"/>
-      <c r="W2" s="3" t="n"/>
-      <c r="X2" s="3" t="n"/>
-      <c r="Y2" s="3" t="n"/>
-    </row>
+    <row r="2" ht="6" customHeight="1"/>
     <row r="4">
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Columns for the actual value with a target line on the same axis. 'vs. target' is a formula you can overwrite.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>Chart title</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>Templates migrated vs. target</t>
         </is>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="C9" s="10" t="inlineStr">
+      <c r="C9" s="9" t="inlineStr">
         <is>
           <t>Migrated</t>
         </is>
       </c>
-      <c r="D9" s="10" t="inlineStr">
+      <c r="D9" s="9" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="E9" s="10" t="inlineStr">
+      <c r="E9" s="9" t="inlineStr">
         <is>
           <t>vs. target</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="11" t="inlineStr">
+      <c r="B10" s="10" t="inlineStr">
         <is>
           <t>Jan</t>
         </is>
       </c>
-      <c r="C10" s="12" t="n">
+      <c r="C10" s="11" t="n">
         <v>182</v>
       </c>
-      <c r="D10" s="12" t="n">
+      <c r="D10" s="11" t="n">
         <v>200</v>
       </c>
-      <c r="E10" s="14">
+      <c r="E10" s="13">
         <f>IF(D10=0,0,C10/D10-1)</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="11" t="inlineStr">
+      <c r="B11" s="10" t="inlineStr">
         <is>
           <t>Feb</t>
         </is>
       </c>
-      <c r="C11" s="12" t="n">
+      <c r="C11" s="11" t="n">
         <v>196</v>
       </c>
-      <c r="D11" s="12" t="n">
+      <c r="D11" s="11" t="n">
         <v>210</v>
       </c>
-      <c r="E11" s="14">
+      <c r="E11" s="13">
         <f>IF(D11=0,0,C11/D11-1)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="11" t="inlineStr">
+      <c r="B12" s="10" t="inlineStr">
         <is>
           <t>Mar</t>
         </is>
       </c>
-      <c r="C12" s="12" t="n">
+      <c r="C12" s="11" t="n">
         <v>228</v>
       </c>
-      <c r="D12" s="12" t="n">
+      <c r="D12" s="11" t="n">
         <v>220</v>
       </c>
-      <c r="E12" s="14">
+      <c r="E12" s="13">
         <f>IF(D12=0,0,C12/D12-1)</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="11" t="inlineStr">
+      <c r="B13" s="10" t="inlineStr">
         <is>
           <t>Apr</t>
         </is>
       </c>
-      <c r="C13" s="12" t="n">
+      <c r="C13" s="11" t="n">
         <v>241</v>
       </c>
-      <c r="D13" s="12" t="n">
+      <c r="D13" s="11" t="n">
         <v>235</v>
       </c>
-      <c r="E13" s="14">
+      <c r="E13" s="13">
         <f>IF(D13=0,0,C13/D13-1)</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="11" t="inlineStr">
+      <c r="B14" s="10" t="inlineStr">
         <is>
           <t>May</t>
         </is>
       </c>
-      <c r="C14" s="12" t="n">
+      <c r="C14" s="11" t="n">
         <v>263</v>
       </c>
-      <c r="D14" s="12" t="n">
+      <c r="D14" s="11" t="n">
         <v>250</v>
       </c>
-      <c r="E14" s="14">
+      <c r="E14" s="13">
         <f>IF(D14=0,0,C14/D14-1)</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="11" t="inlineStr">
+      <c r="B15" s="10" t="inlineStr">
         <is>
           <t>Jun</t>
         </is>
       </c>
-      <c r="C15" s="12" t="n">
+      <c r="C15" s="11" t="n">
         <v>288</v>
       </c>
-      <c r="D15" s="12" t="n">
+      <c r="D15" s="11" t="n">
         <v>265</v>
       </c>
-      <c r="E15" s="14">
+      <c r="E15" s="13">
         <f>IF(D15=0,0,C15/D15-1)</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="7" t="inlineStr">
+      <c r="B16" s="6" t="inlineStr">
         <is>
           <t>Sample data is illustrative. Replace it with your own and cite the source under the table.</t>
         </is>
@@ -5247,7 +5033,7 @@
     <col width="13" customWidth="1" min="29" max="29"/>
   </cols>
   <sheetData>
-    <row r="1" ht="44" customHeight="1">
+    <row r="1" ht="48" customHeight="1">
       <c r="A1" s="1" t="n"/>
       <c r="B1" s="2" t="inlineStr">
         <is>
@@ -5278,129 +5064,103 @@
       <c r="X1" s="1" t="n"/>
       <c r="Y1" s="1" t="n"/>
     </row>
-    <row r="2" ht="4" customHeight="1">
-      <c r="A2" s="3" t="n"/>
-      <c r="B2" s="3" t="n"/>
-      <c r="C2" s="3" t="n"/>
-      <c r="D2" s="3" t="n"/>
-      <c r="E2" s="3" t="n"/>
-      <c r="F2" s="3" t="n"/>
-      <c r="G2" s="3" t="n"/>
-      <c r="H2" s="3" t="n"/>
-      <c r="I2" s="3" t="n"/>
-      <c r="J2" s="3" t="n"/>
-      <c r="K2" s="3" t="n"/>
-      <c r="L2" s="3" t="n"/>
-      <c r="M2" s="3" t="n"/>
-      <c r="N2" s="3" t="n"/>
-      <c r="O2" s="3" t="n"/>
-      <c r="P2" s="3" t="n"/>
-      <c r="Q2" s="3" t="n"/>
-      <c r="R2" s="3" t="n"/>
-      <c r="S2" s="3" t="n"/>
-      <c r="T2" s="3" t="n"/>
-      <c r="U2" s="3" t="n"/>
-      <c r="V2" s="3" t="n"/>
-      <c r="W2" s="3" t="n"/>
-      <c r="X2" s="3" t="n"/>
-      <c r="Y2" s="3" t="n"/>
-    </row>
+    <row r="2" ht="6" customHeight="1"/>
     <row r="4">
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Share of a whole, five slices at most. Order slices from largest to smallest.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>Chart title</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>Where customers start a form</t>
         </is>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>Channel</t>
         </is>
       </c>
-      <c r="C9" s="10" t="inlineStr">
+      <c r="C9" s="9" t="inlineStr">
         <is>
           <t>Share</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="11" t="inlineStr">
+      <c r="B10" s="10" t="inlineStr">
         <is>
           <t>Web portal</t>
         </is>
       </c>
-      <c r="C10" s="15" t="n">
+      <c r="C10" s="14" t="n">
         <v>0.38</v>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="11" t="inlineStr">
+      <c r="B11" s="10" t="inlineStr">
         <is>
           <t>Mobile app</t>
         </is>
       </c>
-      <c r="C11" s="15" t="n">
+      <c r="C11" s="14" t="n">
         <v>0.24</v>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="11" t="inlineStr">
+      <c r="B12" s="10" t="inlineStr">
         <is>
           <t>Agent-assisted</t>
         </is>
       </c>
-      <c r="C12" s="15" t="n">
+      <c r="C12" s="14" t="n">
         <v>0.17</v>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="11" t="inlineStr">
+      <c r="B13" s="10" t="inlineStr">
         <is>
           <t>Email link</t>
         </is>
       </c>
-      <c r="C13" s="15" t="n">
+      <c r="C13" s="14" t="n">
         <v>0.13</v>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="11" t="inlineStr">
+      <c r="B14" s="10" t="inlineStr">
         <is>
           <t>Paper form</t>
         </is>
       </c>
-      <c r="C14" s="15" t="n">
+      <c r="C14" s="14" t="n">
         <v>0.08</v>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="16" t="inlineStr">
+      <c r="B15" s="15" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="C15" s="17">
+      <c r="C15" s="16">
         <f>SUM(C10:C14)</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="7" t="inlineStr">
+      <c r="B16" s="6" t="inlineStr">
         <is>
           <t>Sample data is illustrative. Replace it with your own and cite the source under the table. Shares should total 100%.</t>
         </is>
@@ -5458,7 +5218,7 @@
     <col width="13" customWidth="1" min="29" max="29"/>
   </cols>
   <sheetData>
-    <row r="1" ht="44" customHeight="1">
+    <row r="1" ht="48" customHeight="1">
       <c r="A1" s="1" t="n"/>
       <c r="B1" s="2" t="inlineStr">
         <is>
@@ -5489,153 +5249,127 @@
       <c r="X1" s="1" t="n"/>
       <c r="Y1" s="1" t="n"/>
     </row>
-    <row r="2" ht="4" customHeight="1">
-      <c r="A2" s="3" t="n"/>
-      <c r="B2" s="3" t="n"/>
-      <c r="C2" s="3" t="n"/>
-      <c r="D2" s="3" t="n"/>
-      <c r="E2" s="3" t="n"/>
-      <c r="F2" s="3" t="n"/>
-      <c r="G2" s="3" t="n"/>
-      <c r="H2" s="3" t="n"/>
-      <c r="I2" s="3" t="n"/>
-      <c r="J2" s="3" t="n"/>
-      <c r="K2" s="3" t="n"/>
-      <c r="L2" s="3" t="n"/>
-      <c r="M2" s="3" t="n"/>
-      <c r="N2" s="3" t="n"/>
-      <c r="O2" s="3" t="n"/>
-      <c r="P2" s="3" t="n"/>
-      <c r="Q2" s="3" t="n"/>
-      <c r="R2" s="3" t="n"/>
-      <c r="S2" s="3" t="n"/>
-      <c r="T2" s="3" t="n"/>
-      <c r="U2" s="3" t="n"/>
-      <c r="V2" s="3" t="n"/>
-      <c r="W2" s="3" t="n"/>
-      <c r="X2" s="3" t="n"/>
-      <c r="Y2" s="3" t="n"/>
-    </row>
+    <row r="2" ht="6" customHeight="1"/>
     <row r="4">
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>A formatted table with in-cell bars, for when a chart is too much. Edit the light-blue cells.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="B7" s="9" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>Program</t>
         </is>
       </c>
-      <c r="C7" s="10" t="inlineStr">
+      <c r="C7" s="9" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="D7" s="10" t="inlineStr">
+      <c r="D7" s="9" t="inlineStr">
         <is>
           <t>Actual</t>
         </is>
       </c>
-      <c r="E7" s="10" t="inlineStr">
+      <c r="E7" s="9" t="inlineStr">
         <is>
           <t>vs. target</t>
         </is>
       </c>
-      <c r="F7" s="10" t="inlineStr">
+      <c r="F7" s="9" t="inlineStr">
         <is>
           <t>Progress</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="11" t="inlineStr">
+      <c r="B8" s="10" t="inlineStr">
         <is>
           <t>Template consolidation</t>
         </is>
       </c>
-      <c r="C8" s="12" t="n">
+      <c r="C8" s="11" t="n">
         <v>1200</v>
       </c>
-      <c r="D8" s="12" t="n">
+      <c r="D8" s="11" t="n">
         <v>1056</v>
       </c>
-      <c r="E8" s="14">
+      <c r="E8" s="13">
         <f>IF(C8=0,0,D8/C8-1)</f>
         <v/>
       </c>
-      <c r="F8" s="18">
+      <c r="F8" s="17">
         <f>IF(C8=0,0,MIN(1,D8/C8))</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="11" t="inlineStr">
+      <c r="B9" s="10" t="inlineStr">
         <is>
           <t>Digital adoption</t>
         </is>
       </c>
-      <c r="C9" s="19" t="n">
+      <c r="C9" s="18" t="n">
         <v>0.6</v>
       </c>
-      <c r="D9" s="19" t="n">
+      <c r="D9" s="18" t="n">
         <v>0.54</v>
       </c>
-      <c r="E9" s="14">
+      <c r="E9" s="13">
         <f>IF(C9=0,0,D9/C9-1)</f>
         <v/>
       </c>
-      <c r="F9" s="18">
+      <c r="F9" s="17">
         <f>IF(C9=0,0,MIN(1,D9/C9))</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="11" t="inlineStr">
+      <c r="B10" s="10" t="inlineStr">
         <is>
           <t>Straight-through processing</t>
         </is>
       </c>
-      <c r="C10" s="19" t="n">
+      <c r="C10" s="18" t="n">
         <v>0.85</v>
       </c>
-      <c r="D10" s="19" t="n">
+      <c r="D10" s="18" t="n">
         <v>0.8100000000000001</v>
       </c>
-      <c r="E10" s="14">
+      <c r="E10" s="13">
         <f>IF(C10=0,0,D10/C10-1)</f>
         <v/>
       </c>
-      <c r="F10" s="18">
+      <c r="F10" s="17">
         <f>IF(C10=0,0,MIN(1,D10/C10))</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="11" t="inlineStr">
+      <c r="B11" s="10" t="inlineStr">
         <is>
           <t>Self-service forms live</t>
         </is>
       </c>
-      <c r="C11" s="12" t="n">
+      <c r="C11" s="11" t="n">
         <v>40</v>
       </c>
-      <c r="D11" s="12" t="n">
+      <c r="D11" s="11" t="n">
         <v>46</v>
       </c>
-      <c r="E11" s="14">
+      <c r="E11" s="13">
         <f>IF(C11=0,0,D11/C11-1)</f>
         <v/>
       </c>
-      <c r="F11" s="18">
+      <c r="F11" s="17">
         <f>IF(C11=0,0,MIN(1,D11/C11))</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="7" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>Sample data is illustrative. Replace it with your own and cite the source under the table. 'vs. target' and 'Progress' are formulas.</t>
         </is>

</xml_diff>

<commit_message>
Excel templates: progress bars, larger chart text, roomier labels and keys
Table tab: solid progress bars on a light-gray track with the percentage to the left,
a gap column after 'vs. target', and numbers inset from the cell edge. Charts: larger
titles, axes, legends and value labels; category labels and bar values sit off the
axis and bars; legend entries get padding; the doughnut key moves to the top right
under a 'Key' heading, with the lead slice's label reversed out. The header banner
ends at column S and is backed by its end color. Ignore Office lock files.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/site/assets/downloads/SmartCommunications_Excel_Chart_Templates.xlsx
+++ b/site/assets/downloads/SmartCommunications_Excel_Chart_Templates.xlsx
@@ -25,12 +25,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="0&quot;%&quot;"/>
     <numFmt numFmtId="165" formatCode="+0.0%;-0.0%;0.0%"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
+    <numFmt numFmtId="167" formatCode=";;;"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -79,12 +80,23 @@
     </font>
     <font>
       <name val="Segoe UI"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="1"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
       <b val="1"/>
       <color rgb="00183958"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00183958"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -93,12 +105,22 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00326EEF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EFF4F9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="000E2030"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EFF4F9"/>
+        <fgColor rgb="00E3E7EC"/>
       </patternFill>
     </fill>
     <fill>
@@ -132,7 +154,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -145,11 +167,17 @@
         <color rgb="00D0DEEC"/>
       </bottom>
     </border>
+    <border/>
+    <border>
+      <bottom style="thick">
+        <color rgb="00FFFFFF"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -160,43 +188,55 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" indent="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" indent="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" indent="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="165" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
+      <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
+    <xf numFmtId="167" fontId="0" fillId="5" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="9" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -304,7 +344,7 @@
         <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
         <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
-            <a:defRPr sz="1400" b="1">
+            <a:defRPr sz="1800" b="1">
               <a:solidFill>
                 <a:srgbClr val="0E2030"/>
               </a:solidFill>
@@ -314,7 +354,7 @@
           <a:r>
             <a:t/>
           </a:r>
-          <a:endParaRPr sz="1400" b="1">
+          <a:endParaRPr sz="1800" b="1">
             <a:solidFill>
               <a:srgbClr val="0E2030"/>
             </a:solidFill>
@@ -332,7 +372,13 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Column'!C9</f>
+              <f>'Column'!$C$8</f>
+              <strCache>
+                <ptCount val="1"/>
+                <pt idx="0">
+                  <v xml:space="preserve">  Email     </v>
+                </pt>
+              </strCache>
             </strRef>
           </tx>
           <spPr>
@@ -360,7 +406,13 @@
           <order val="1"/>
           <tx>
             <strRef>
-              <f>'Column'!D9</f>
+              <f>'Column'!$D$8</f>
+              <strCache>
+                <ptCount val="1"/>
+                <pt idx="0">
+                  <v xml:space="preserve">  Print     </v>
+                </pt>
+              </strCache>
             </strRef>
           </tx>
           <spPr>
@@ -388,7 +440,13 @@
           <order val="2"/>
           <tx>
             <strRef>
-              <f>'Column'!E9</f>
+              <f>'Column'!$E$8</f>
+              <strCache>
+                <ptCount val="1"/>
+                <pt idx="0">
+                  <v xml:space="preserve">  SMS     </v>
+                </pt>
+              </strCache>
             </strRef>
           </tx>
           <spPr>
@@ -416,7 +474,13 @@
           <order val="3"/>
           <tx>
             <strRef>
-              <f>'Column'!F9</f>
+              <f>'Column'!$F$8</f>
+              <strCache>
+                <ptCount val="1"/>
+                <pt idx="0">
+                  <v xml:space="preserve">  Portal     </v>
+                </pt>
+              </strCache>
             </strRef>
           </tx>
           <spPr>
@@ -444,7 +508,13 @@
           <order val="4"/>
           <tx>
             <strRef>
-              <f>'Column'!G9</f>
+              <f>'Column'!$G$8</f>
+              <strCache>
+                <ptCount val="1"/>
+                <pt idx="0">
+                  <v xml:space="preserve">  App     </v>
+                </pt>
+              </strCache>
             </strRef>
           </tx>
           <spPr>
@@ -493,7 +563,7 @@
           <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
-              <a:defRPr sz="900" b="0">
+              <a:defRPr sz="1300" b="0">
                 <a:solidFill>
                   <a:srgbClr val="677C91"/>
                 </a:solidFill>
@@ -503,7 +573,7 @@
             <a:r>
               <a:t/>
             </a:r>
-            <a:endParaRPr sz="900" b="0">
+            <a:endParaRPr sz="1300" b="0">
               <a:solidFill>
                 <a:srgbClr val="677C91"/>
               </a:solidFill>
@@ -512,7 +582,7 @@
           </a:p>
         </txPr>
         <crossAx val="100"/>
-        <lblOffset val="100"/>
+        <lblOffset val="200"/>
       </catAx>
       <valAx>
         <axId val="100"/>
@@ -544,7 +614,7 @@
           <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
-              <a:defRPr sz="900" b="0">
+              <a:defRPr sz="1300" b="0">
                 <a:solidFill>
                   <a:srgbClr val="677C91"/>
                 </a:solidFill>
@@ -554,7 +624,7 @@
             <a:r>
               <a:t/>
             </a:r>
-            <a:endParaRPr sz="900" b="0">
+            <a:endParaRPr sz="1300" b="0">
               <a:solidFill>
                 <a:srgbClr val="677C91"/>
               </a:solidFill>
@@ -579,7 +649,7 @@
         <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
         <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
-            <a:defRPr sz="900" b="0">
+            <a:defRPr sz="1400" b="0">
               <a:solidFill>
                 <a:srgbClr val="183958"/>
               </a:solidFill>
@@ -589,7 +659,7 @@
           <a:r>
             <a:t/>
           </a:r>
-          <a:endParaRPr sz="900" b="0">
+          <a:endParaRPr sz="1400" b="0">
             <a:solidFill>
               <a:srgbClr val="183958"/>
             </a:solidFill>
@@ -644,7 +714,7 @@
         <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
         <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
-            <a:defRPr sz="1400" b="1">
+            <a:defRPr sz="1800" b="1">
               <a:solidFill>
                 <a:srgbClr val="FFFFFF"/>
               </a:solidFill>
@@ -654,7 +724,7 @@
           <a:r>
             <a:t/>
           </a:r>
-          <a:endParaRPr sz="1400" b="1">
+          <a:endParaRPr sz="1800" b="1">
             <a:solidFill>
               <a:srgbClr val="FFFFFF"/>
             </a:solidFill>
@@ -672,7 +742,13 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Column (dark)'!C9</f>
+              <f>'Column (dark)'!$C$8</f>
+              <strCache>
+                <ptCount val="1"/>
+                <pt idx="0">
+                  <v xml:space="preserve">  Email     </v>
+                </pt>
+              </strCache>
             </strRef>
           </tx>
           <spPr>
@@ -700,7 +776,13 @@
           <order val="1"/>
           <tx>
             <strRef>
-              <f>'Column (dark)'!D9</f>
+              <f>'Column (dark)'!$D$8</f>
+              <strCache>
+                <ptCount val="1"/>
+                <pt idx="0">
+                  <v xml:space="preserve">  Print     </v>
+                </pt>
+              </strCache>
             </strRef>
           </tx>
           <spPr>
@@ -728,7 +810,13 @@
           <order val="2"/>
           <tx>
             <strRef>
-              <f>'Column (dark)'!E9</f>
+              <f>'Column (dark)'!$E$8</f>
+              <strCache>
+                <ptCount val="1"/>
+                <pt idx="0">
+                  <v xml:space="preserve">  SMS     </v>
+                </pt>
+              </strCache>
             </strRef>
           </tx>
           <spPr>
@@ -756,7 +844,13 @@
           <order val="3"/>
           <tx>
             <strRef>
-              <f>'Column (dark)'!F9</f>
+              <f>'Column (dark)'!$F$8</f>
+              <strCache>
+                <ptCount val="1"/>
+                <pt idx="0">
+                  <v xml:space="preserve">  Portal     </v>
+                </pt>
+              </strCache>
             </strRef>
           </tx>
           <spPr>
@@ -805,7 +899,7 @@
           <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
-              <a:defRPr sz="900" b="0">
+              <a:defRPr sz="1300" b="0">
                 <a:solidFill>
                   <a:srgbClr val="FFFFFF"/>
                 </a:solidFill>
@@ -815,7 +909,7 @@
             <a:r>
               <a:t/>
             </a:r>
-            <a:endParaRPr sz="900" b="0">
+            <a:endParaRPr sz="1300" b="0">
               <a:solidFill>
                 <a:srgbClr val="FFFFFF"/>
               </a:solidFill>
@@ -824,7 +918,7 @@
           </a:p>
         </txPr>
         <crossAx val="100"/>
-        <lblOffset val="100"/>
+        <lblOffset val="200"/>
       </catAx>
       <valAx>
         <axId val="100"/>
@@ -856,7 +950,7 @@
           <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
-              <a:defRPr sz="900" b="0">
+              <a:defRPr sz="1300" b="0">
                 <a:solidFill>
                   <a:srgbClr val="FFFFFF"/>
                 </a:solidFill>
@@ -866,7 +960,7 @@
             <a:r>
               <a:t/>
             </a:r>
-            <a:endParaRPr sz="900" b="0">
+            <a:endParaRPr sz="1300" b="0">
               <a:solidFill>
                 <a:srgbClr val="FFFFFF"/>
               </a:solidFill>
@@ -891,7 +985,7 @@
         <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
         <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
-            <a:defRPr sz="900" b="0">
+            <a:defRPr sz="1400" b="0">
               <a:solidFill>
                 <a:srgbClr val="FFFFFF"/>
               </a:solidFill>
@@ -901,7 +995,7 @@
           <a:r>
             <a:t/>
           </a:r>
-          <a:endParaRPr sz="900" b="0">
+          <a:endParaRPr sz="1400" b="0">
             <a:solidFill>
               <a:srgbClr val="FFFFFF"/>
             </a:solidFill>
@@ -956,7 +1050,7 @@
         <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
         <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
-            <a:defRPr sz="1400" b="1">
+            <a:defRPr sz="1800" b="1">
               <a:solidFill>
                 <a:srgbClr val="0E2030"/>
               </a:solidFill>
@@ -966,7 +1060,7 @@
           <a:r>
             <a:t/>
           </a:r>
-          <a:endParaRPr sz="1400" b="1">
+          <a:endParaRPr sz="1800" b="1">
             <a:solidFill>
               <a:srgbClr val="0E2030"/>
             </a:solidFill>
@@ -997,11 +1091,12 @@
             </a:ln>
           </spPr>
           <dLbls>
+            <numFmt formatCode="&quot;  &quot;#,##0"/>
             <txPr>
               <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
               <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
-                  <a:defRPr sz="900" b="1">
+                  <a:defRPr sz="1600" b="1">
                     <a:solidFill>
                       <a:srgbClr val="183958"/>
                     </a:solidFill>
@@ -1011,7 +1106,7 @@
                 <a:r>
                   <a:t/>
                 </a:r>
-                <a:endParaRPr sz="900" b="1">
+                <a:endParaRPr sz="1600" b="1">
                   <a:solidFill>
                     <a:srgbClr val="183958"/>
                   </a:solidFill>
@@ -1062,9 +1157,9 @@
           <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
-              <a:defRPr sz="900" b="0">
+              <a:defRPr sz="1500" b="0">
                 <a:solidFill>
-                  <a:srgbClr val="677C91"/>
+                  <a:srgbClr val="183958"/>
                 </a:solidFill>
                 <a:latin typeface="Segoe UI"/>
               </a:defRPr>
@@ -1072,16 +1167,16 @@
             <a:r>
               <a:t/>
             </a:r>
-            <a:endParaRPr sz="900" b="0">
+            <a:endParaRPr sz="1500" b="0">
               <a:solidFill>
-                <a:srgbClr val="677C91"/>
+                <a:srgbClr val="183958"/>
               </a:solidFill>
               <a:latin typeface="Segoe UI"/>
             </a:endParaRPr>
           </a:p>
         </txPr>
         <crossAx val="100"/>
-        <lblOffset val="100"/>
+        <lblOffset val="200"/>
       </catAx>
       <valAx>
         <axId val="100"/>
@@ -1103,7 +1198,7 @@
           <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
-              <a:defRPr sz="900" b="0">
+              <a:defRPr sz="1300" b="0">
                 <a:solidFill>
                   <a:srgbClr val="677C91"/>
                 </a:solidFill>
@@ -1113,7 +1208,7 @@
             <a:r>
               <a:t/>
             </a:r>
-            <a:endParaRPr sz="900" b="0">
+            <a:endParaRPr sz="1300" b="0">
               <a:solidFill>
                 <a:srgbClr val="677C91"/>
               </a:solidFill>
@@ -1177,7 +1272,7 @@
         <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
         <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
-            <a:defRPr sz="1400" b="1">
+            <a:defRPr sz="1800" b="1">
               <a:solidFill>
                 <a:srgbClr val="0E2030"/>
               </a:solidFill>
@@ -1187,7 +1282,7 @@
           <a:r>
             <a:t/>
           </a:r>
-          <a:endParaRPr sz="1400" b="1">
+          <a:endParaRPr sz="1800" b="1">
             <a:solidFill>
               <a:srgbClr val="0E2030"/>
             </a:solidFill>
@@ -1205,7 +1300,13 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Stacked'!C9</f>
+              <f>'Stacked'!$C$8</f>
+              <strCache>
+                <ptCount val="1"/>
+                <pt idx="0">
+                  <v xml:space="preserve">  Email     </v>
+                </pt>
+              </strCache>
             </strRef>
           </tx>
           <spPr>
@@ -1235,7 +1336,13 @@
           <order val="1"/>
           <tx>
             <strRef>
-              <f>'Stacked'!D9</f>
+              <f>'Stacked'!$D$8</f>
+              <strCache>
+                <ptCount val="1"/>
+                <pt idx="0">
+                  <v xml:space="preserve">  Portal     </v>
+                </pt>
+              </strCache>
             </strRef>
           </tx>
           <spPr>
@@ -1265,7 +1372,13 @@
           <order val="2"/>
           <tx>
             <strRef>
-              <f>'Stacked'!E9</f>
+              <f>'Stacked'!$E$8</f>
+              <strCache>
+                <ptCount val="1"/>
+                <pt idx="0">
+                  <v xml:space="preserve">  SMS     </v>
+                </pt>
+              </strCache>
             </strRef>
           </tx>
           <spPr>
@@ -1295,7 +1408,13 @@
           <order val="3"/>
           <tx>
             <strRef>
-              <f>'Stacked'!F9</f>
+              <f>'Stacked'!$F$8</f>
+              <strCache>
+                <ptCount val="1"/>
+                <pt idx="0">
+                  <v xml:space="preserve">  Print     </v>
+                </pt>
+              </strCache>
             </strRef>
           </tx>
           <spPr>
@@ -1346,7 +1465,7 @@
           <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
-              <a:defRPr sz="900" b="0">
+              <a:defRPr sz="1300" b="0">
                 <a:solidFill>
                   <a:srgbClr val="677C91"/>
                 </a:solidFill>
@@ -1356,7 +1475,7 @@
             <a:r>
               <a:t/>
             </a:r>
-            <a:endParaRPr sz="900" b="0">
+            <a:endParaRPr sz="1300" b="0">
               <a:solidFill>
                 <a:srgbClr val="677C91"/>
               </a:solidFill>
@@ -1365,7 +1484,7 @@
           </a:p>
         </txPr>
         <crossAx val="100"/>
-        <lblOffset val="100"/>
+        <lblOffset val="200"/>
       </catAx>
       <valAx>
         <axId val="100"/>
@@ -1397,7 +1516,7 @@
           <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
-              <a:defRPr sz="900" b="0">
+              <a:defRPr sz="1300" b="0">
                 <a:solidFill>
                   <a:srgbClr val="677C91"/>
                 </a:solidFill>
@@ -1407,7 +1526,7 @@
             <a:r>
               <a:t/>
             </a:r>
-            <a:endParaRPr sz="900" b="0">
+            <a:endParaRPr sz="1300" b="0">
               <a:solidFill>
                 <a:srgbClr val="677C91"/>
               </a:solidFill>
@@ -1432,7 +1551,7 @@
         <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
         <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
-            <a:defRPr sz="900" b="0">
+            <a:defRPr sz="1400" b="0">
               <a:solidFill>
                 <a:srgbClr val="183958"/>
               </a:solidFill>
@@ -1442,7 +1561,7 @@
           <a:r>
             <a:t/>
           </a:r>
-          <a:endParaRPr sz="900" b="0">
+          <a:endParaRPr sz="1400" b="0">
             <a:solidFill>
               <a:srgbClr val="183958"/>
             </a:solidFill>
@@ -1497,7 +1616,7 @@
         <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
         <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
-            <a:defRPr sz="1400" b="1">
+            <a:defRPr sz="1800" b="1">
               <a:solidFill>
                 <a:srgbClr val="0E2030"/>
               </a:solidFill>
@@ -1507,7 +1626,7 @@
           <a:r>
             <a:t/>
           </a:r>
-          <a:endParaRPr sz="1400" b="1">
+          <a:endParaRPr sz="1800" b="1">
             <a:solidFill>
               <a:srgbClr val="0E2030"/>
             </a:solidFill>
@@ -1524,7 +1643,13 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Line'!C9</f>
+              <f>'Line'!$C$8</f>
+              <strCache>
+                <ptCount val="1"/>
+                <pt idx="0">
+                  <v xml:space="preserve">  2026     </v>
+                </pt>
+              </strCache>
             </strRef>
           </tx>
           <spPr>
@@ -1560,7 +1685,13 @@
           <order val="1"/>
           <tx>
             <strRef>
-              <f>'Line'!D9</f>
+              <f>'Line'!$D$8</f>
+              <strCache>
+                <ptCount val="1"/>
+                <pt idx="0">
+                  <v xml:space="preserve">  2025     </v>
+                </pt>
+              </strCache>
             </strRef>
           </tx>
           <spPr>
@@ -1615,7 +1746,7 @@
           <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
-              <a:defRPr sz="900" b="0">
+              <a:defRPr sz="1300" b="0">
                 <a:solidFill>
                   <a:srgbClr val="677C91"/>
                 </a:solidFill>
@@ -1625,7 +1756,7 @@
             <a:r>
               <a:t/>
             </a:r>
-            <a:endParaRPr sz="900" b="0">
+            <a:endParaRPr sz="1300" b="0">
               <a:solidFill>
                 <a:srgbClr val="677C91"/>
               </a:solidFill>
@@ -1634,7 +1765,7 @@
           </a:p>
         </txPr>
         <crossAx val="100"/>
-        <lblOffset val="100"/>
+        <lblOffset val="300"/>
       </catAx>
       <valAx>
         <axId val="100"/>
@@ -1666,7 +1797,7 @@
           <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
-              <a:defRPr sz="900" b="0">
+              <a:defRPr sz="1300" b="0">
                 <a:solidFill>
                   <a:srgbClr val="677C91"/>
                 </a:solidFill>
@@ -1676,7 +1807,7 @@
             <a:r>
               <a:t/>
             </a:r>
-            <a:endParaRPr sz="900" b="0">
+            <a:endParaRPr sz="1300" b="0">
               <a:solidFill>
                 <a:srgbClr val="677C91"/>
               </a:solidFill>
@@ -1701,7 +1832,7 @@
         <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
         <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
-            <a:defRPr sz="900" b="0">
+            <a:defRPr sz="1400" b="0">
               <a:solidFill>
                 <a:srgbClr val="183958"/>
               </a:solidFill>
@@ -1711,7 +1842,7 @@
           <a:r>
             <a:t/>
           </a:r>
-          <a:endParaRPr sz="900" b="0">
+          <a:endParaRPr sz="1400" b="0">
             <a:solidFill>
               <a:srgbClr val="183958"/>
             </a:solidFill>
@@ -1766,7 +1897,7 @@
         <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
         <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
-            <a:defRPr sz="1400" b="1">
+            <a:defRPr sz="1800" b="1">
               <a:solidFill>
                 <a:srgbClr val="0E2030"/>
               </a:solidFill>
@@ -1776,7 +1907,7 @@
           <a:r>
             <a:t/>
           </a:r>
-          <a:endParaRPr sz="1400" b="1">
+          <a:endParaRPr sz="1800" b="1">
             <a:solidFill>
               <a:srgbClr val="0E2030"/>
             </a:solidFill>
@@ -1794,7 +1925,13 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Combo'!C9</f>
+              <f>'Combo'!$C$8</f>
+              <strCache>
+                <ptCount val="1"/>
+                <pt idx="0">
+                  <v xml:space="preserve">  Migrated     </v>
+                </pt>
+              </strCache>
             </strRef>
           </tx>
           <spPr>
@@ -1828,7 +1965,13 @@
           <order val="1"/>
           <tx>
             <strRef>
-              <f>'Combo'!D9</f>
+              <f>'Combo'!$D$8</f>
+              <strCache>
+                <ptCount val="1"/>
+                <pt idx="0">
+                  <v xml:space="preserve">  Target     </v>
+                </pt>
+              </strCache>
             </strRef>
           </tx>
           <spPr>
@@ -1884,7 +2027,7 @@
           <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
-              <a:defRPr sz="900" b="0">
+              <a:defRPr sz="1300" b="0">
                 <a:solidFill>
                   <a:srgbClr val="677C91"/>
                 </a:solidFill>
@@ -1894,7 +2037,7 @@
             <a:r>
               <a:t/>
             </a:r>
-            <a:endParaRPr sz="900" b="0">
+            <a:endParaRPr sz="1300" b="0">
               <a:solidFill>
                 <a:srgbClr val="677C91"/>
               </a:solidFill>
@@ -1903,7 +2046,7 @@
           </a:p>
         </txPr>
         <crossAx val="100"/>
-        <lblOffset val="100"/>
+        <lblOffset val="200"/>
       </catAx>
       <valAx>
         <axId val="100"/>
@@ -1935,7 +2078,7 @@
           <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
-              <a:defRPr sz="900" b="0">
+              <a:defRPr sz="1300" b="0">
                 <a:solidFill>
                   <a:srgbClr val="677C91"/>
                 </a:solidFill>
@@ -1945,7 +2088,7 @@
             <a:r>
               <a:t/>
             </a:r>
-            <a:endParaRPr sz="900" b="0">
+            <a:endParaRPr sz="1300" b="0">
               <a:solidFill>
                 <a:srgbClr val="677C91"/>
               </a:solidFill>
@@ -1970,7 +2113,7 @@
         <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
         <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
-            <a:defRPr sz="900" b="0">
+            <a:defRPr sz="1400" b="0">
               <a:solidFill>
                 <a:srgbClr val="183958"/>
               </a:solidFill>
@@ -1980,7 +2123,7 @@
           <a:r>
             <a:t/>
           </a:r>
-          <a:endParaRPr sz="900" b="0">
+          <a:endParaRPr sz="1400" b="0">
             <a:solidFill>
               <a:srgbClr val="183958"/>
             </a:solidFill>
@@ -2035,7 +2178,7 @@
         <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
         <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
-            <a:defRPr sz="1400" b="1">
+            <a:defRPr sz="1800" b="1">
               <a:solidFill>
                 <a:srgbClr val="0E2030"/>
               </a:solidFill>
@@ -2045,7 +2188,7 @@
           <a:r>
             <a:t/>
           </a:r>
-          <a:endParaRPr sz="1400" b="1">
+          <a:endParaRPr sz="1800" b="1">
             <a:solidFill>
               <a:srgbClr val="0E2030"/>
             </a:solidFill>
@@ -2055,6 +2198,18 @@
       </txPr>
     </title>
     <plotArea>
+      <layout>
+        <manualLayout>
+          <xMode val="edge"/>
+          <yMode val="edge"/>
+          <wMode val="factor"/>
+          <hMode val="factor"/>
+          <x val="0.04"/>
+          <y val="0.17"/>
+          <w val="0.52"/>
+          <h val="0.78"/>
+        </manualLayout>
+      </layout>
       <doughnutChart>
         <varyColors val="1"/>
         <ser>
@@ -2147,9 +2302,9 @@
                 <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
                 <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
-                    <a:defRPr sz="1000" b="1">
+                    <a:defRPr sz="1600" b="1">
                       <a:solidFill>
-                        <a:srgbClr val="0E2030"/>
+                        <a:srgbClr val="FFFFFF"/>
                       </a:solidFill>
                       <a:latin typeface="Segoe UI"/>
                     </a:defRPr>
@@ -2157,9 +2312,9 @@
                   <a:r>
                     <a:t/>
                   </a:r>
-                  <a:endParaRPr sz="1000" b="1">
+                  <a:endParaRPr sz="1600" b="1">
                     <a:solidFill>
-                      <a:srgbClr val="0E2030"/>
+                      <a:srgbClr val="FFFFFF"/>
                     </a:solidFill>
                     <a:latin typeface="Segoe UI"/>
                   </a:endParaRPr>
@@ -2177,7 +2332,7 @@
                 <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
                 <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
-                    <a:defRPr sz="1000" b="1">
+                    <a:defRPr sz="1600" b="1">
                       <a:solidFill>
                         <a:srgbClr val="FFFFFF"/>
                       </a:solidFill>
@@ -2187,7 +2342,7 @@
                   <a:r>
                     <a:t/>
                   </a:r>
-                  <a:endParaRPr sz="1000" b="1">
+                  <a:endParaRPr sz="1600" b="1">
                     <a:solidFill>
                       <a:srgbClr val="FFFFFF"/>
                     </a:solidFill>
@@ -2207,7 +2362,7 @@
                 <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
                 <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
-                    <a:defRPr sz="1000" b="1">
+                    <a:defRPr sz="1600" b="1">
                       <a:solidFill>
                         <a:srgbClr val="0E2030"/>
                       </a:solidFill>
@@ -2217,7 +2372,7 @@
                   <a:r>
                     <a:t/>
                   </a:r>
-                  <a:endParaRPr sz="1000" b="1">
+                  <a:endParaRPr sz="1600" b="1">
                     <a:solidFill>
                       <a:srgbClr val="0E2030"/>
                     </a:solidFill>
@@ -2237,7 +2392,7 @@
                 <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
                 <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
-                    <a:defRPr sz="1000" b="1">
+                    <a:defRPr sz="1600" b="1">
                       <a:solidFill>
                         <a:srgbClr val="FFFFFF"/>
                       </a:solidFill>
@@ -2247,7 +2402,7 @@
                   <a:r>
                     <a:t/>
                   </a:r>
-                  <a:endParaRPr sz="1000" b="1">
+                  <a:endParaRPr sz="1600" b="1">
                     <a:solidFill>
                       <a:srgbClr val="FFFFFF"/>
                     </a:solidFill>
@@ -2267,7 +2422,7 @@
                 <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
                 <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
-                    <a:defRPr sz="1000" b="1">
+                    <a:defRPr sz="1600" b="1">
                       <a:solidFill>
                         <a:srgbClr val="0E2030"/>
                       </a:solidFill>
@@ -2277,7 +2432,7 @@
                   <a:r>
                     <a:t/>
                   </a:r>
-                  <a:endParaRPr sz="1000" b="1">
+                  <a:endParaRPr sz="1600" b="1">
                     <a:solidFill>
                       <a:srgbClr val="0E2030"/>
                     </a:solidFill>
@@ -2295,7 +2450,7 @@
               <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
               <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
-                  <a:defRPr sz="1000" b="1">
+                  <a:defRPr sz="1600" b="1">
                     <a:solidFill>
                       <a:srgbClr val="0E2030"/>
                     </a:solidFill>
@@ -2305,7 +2460,7 @@
                 <a:r>
                   <a:t/>
                 </a:r>
-                <a:endParaRPr sz="1000" b="1">
+                <a:endParaRPr sz="1600" b="1">
                   <a:solidFill>
                     <a:srgbClr val="0E2030"/>
                   </a:solidFill>
@@ -2343,12 +2498,24 @@
     </plotArea>
     <legend>
       <legendPos val="r"/>
+      <layout>
+        <manualLayout>
+          <xMode val="edge"/>
+          <yMode val="edge"/>
+          <wMode val="factor"/>
+          <hMode val="factor"/>
+          <x val="0.5600000000000001"/>
+          <y val="0.27"/>
+          <w val="0.24"/>
+          <h val="0.4"/>
+        </manualLayout>
+      </layout>
       <overlay val="0"/>
       <txPr>
         <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
         <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
-            <a:defRPr sz="900" b="0">
+            <a:defRPr sz="1400" b="0">
               <a:solidFill>
                 <a:srgbClr val="183958"/>
               </a:solidFill>
@@ -2358,7 +2525,7 @@
           <a:r>
             <a:t/>
           </a:r>
-          <a:endParaRPr sz="900" b="0">
+          <a:endParaRPr sz="1400" b="0">
             <a:solidFill>
               <a:srgbClr val="183958"/>
             </a:solidFill>
@@ -2379,6 +2546,7 @@
       <a:prstDash val="solid"/>
     </a:ln>
   </spPr>
+  <userShapes xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rIdScKey"/>
 </chartSpace>
 </file>
 
@@ -2391,7 +2559,7 @@
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="23936325" cy="609600"/>
+    <ext cx="18230850" cy="609600"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -2421,7 +2589,7 @@
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="25946100" cy="609600"/>
+    <ext cx="20240625" cy="609600"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -2473,7 +2641,7 @@
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="23660100" cy="609600"/>
+    <ext cx="17954625" cy="609600"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>
@@ -2525,7 +2693,7 @@
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="23660100" cy="609600"/>
+    <ext cx="17954625" cy="609600"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>
@@ -2577,7 +2745,7 @@
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="23660100" cy="609600"/>
+    <ext cx="17954625" cy="609600"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>
@@ -2629,7 +2797,7 @@
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="23660100" cy="609600"/>
+    <ext cx="17954625" cy="609600"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>
@@ -2681,7 +2849,7 @@
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="23660100" cy="609600"/>
+    <ext cx="17954625" cy="609600"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>
@@ -2733,7 +2901,7 @@
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="24079200" cy="609600"/>
+    <ext cx="18373725" cy="609600"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>
@@ -2785,7 +2953,7 @@
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="23660100" cy="609600"/>
+    <ext cx="17954625" cy="609600"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>
@@ -2815,7 +2983,7 @@
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="24212550" cy="609600"/>
+    <ext cx="19069050" cy="609600"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -2834,6 +3002,52 @@
     <clientData/>
   </oneCellAnchor>
 </wsDr>
+</file>
+
+<file path=xl/drawings/sc_chart_key1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:userShapes xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing">
+  <cdr:relSizeAnchor>
+    <cdr:from>
+      <cdr:x>0.56</cdr:x>
+      <cdr:y>0.2</cdr:y>
+    </cdr:from>
+    <cdr:to>
+      <cdr:x>0.76</cdr:x>
+      <cdr:y>0.27</cdr:y>
+    </cdr:to>
+    <cdr:sp macro="" textlink="">
+      <cdr:nvSpPr>
+        <cdr:cNvPr id="2" name="Key"/>
+        <cdr:cNvSpPr txBox="1"/>
+      </cdr:nvSpPr>
+      <cdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </cdr:spPr>
+      <cdr:txBody>
+        <a:bodyPr wrap="none" lIns="0" tIns="0" rIns="0" bIns="0" anchor="b"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1400" b="1">
+              <a:solidFill>
+                <a:srgbClr val="0E2030"/>
+              </a:solidFill>
+              <a:latin typeface="Segoe UI"/>
+            </a:rPr>
+            <a:t>Key</a:t>
+          </a:r>
+        </a:p>
+      </cdr:txBody>
+    </cdr:sp>
+  </cdr:relSizeAnchor>
+</c:userShapes>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3126,7 +3340,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Y21"/>
+  <dimension ref="A1:S21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.5" customWidth="1" min="1" max="1"/>
@@ -3184,12 +3398,6 @@
       <c r="Q1" s="1" t="n"/>
       <c r="R1" s="1" t="n"/>
       <c r="S1" s="1" t="n"/>
-      <c r="T1" s="1" t="n"/>
-      <c r="U1" s="1" t="n"/>
-      <c r="V1" s="1" t="n"/>
-      <c r="W1" s="1" t="n"/>
-      <c r="X1" s="1" t="n"/>
-      <c r="Y1" s="1" t="n"/>
     </row>
     <row r="2" ht="6" customHeight="1"/>
     <row r="4">
@@ -3314,7 +3522,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Y20"/>
+  <dimension ref="A1:S20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.5" customWidth="1" min="1" max="1"/>
@@ -3372,12 +3580,6 @@
       <c r="Q1" s="1" t="n"/>
       <c r="R1" s="1" t="n"/>
       <c r="S1" s="1" t="n"/>
-      <c r="T1" s="1" t="n"/>
-      <c r="U1" s="1" t="n"/>
-      <c r="V1" s="1" t="n"/>
-      <c r="W1" s="1" t="n"/>
-      <c r="X1" s="1" t="n"/>
-      <c r="Y1" s="1" t="n"/>
     </row>
     <row r="2" ht="6" customHeight="1"/>
     <row r="4">
@@ -3388,188 +3590,188 @@
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="19" t="inlineStr">
+      <c r="B7" s="25" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="C7" s="19" t="inlineStr">
+      <c r="C7" s="25" t="inlineStr">
         <is>
           <t>Color</t>
         </is>
       </c>
-      <c r="D7" s="19" t="inlineStr">
+      <c r="D7" s="25" t="inlineStr">
         <is>
           <t>HEX</t>
         </is>
       </c>
-      <c r="E7" s="19" t="inlineStr">
+      <c r="E7" s="25" t="inlineStr">
         <is>
           <t>Swatch</t>
         </is>
       </c>
-      <c r="F7" s="19" t="inlineStr">
+      <c r="F7" s="25" t="inlineStr">
         <is>
           <t>Use for</t>
         </is>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="B8" s="20" t="inlineStr">
+      <c r="B8" s="26" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="C8" s="20" t="inlineStr">
+      <c r="C8" s="26" t="inlineStr">
         <is>
           <t>Dodger</t>
         </is>
       </c>
-      <c r="D8" s="20" t="inlineStr">
+      <c r="D8" s="26" t="inlineStr">
         <is>
           <t>#0094FF</t>
         </is>
       </c>
-      <c r="E8" s="21" t="inlineStr"/>
-      <c r="F8" s="20" t="inlineStr">
+      <c r="E8" s="27" t="inlineStr"/>
+      <c r="F8" s="26" t="inlineStr">
         <is>
           <t>Lead series. Single-series charts use only this</t>
         </is>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="B9" s="20" t="inlineStr">
+      <c r="B9" s="26" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="C9" s="20" t="inlineStr">
+      <c r="C9" s="26" t="inlineStr">
         <is>
           <t>Indigo Dark</t>
         </is>
       </c>
-      <c r="D9" s="20" t="inlineStr">
+      <c r="D9" s="26" t="inlineStr">
         <is>
           <t>#661DEE</t>
         </is>
       </c>
-      <c r="E9" s="22" t="inlineStr"/>
-      <c r="F9" s="20" t="inlineStr">
+      <c r="E9" s="28" t="inlineStr"/>
+      <c r="F9" s="26" t="inlineStr">
         <is>
           <t>Second series, targets and comparisons</t>
         </is>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="B10" s="20" t="inlineStr">
+      <c r="B10" s="26" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="C10" s="20" t="inlineStr">
+      <c r="C10" s="26" t="inlineStr">
         <is>
           <t>Dodger Light</t>
         </is>
       </c>
-      <c r="D10" s="20" t="inlineStr">
+      <c r="D10" s="26" t="inlineStr">
         <is>
           <t>#57B8FF</t>
         </is>
       </c>
-      <c r="E10" s="23" t="inlineStr"/>
-      <c r="F10" s="20" t="inlineStr">
+      <c r="E10" s="29" t="inlineStr"/>
+      <c r="F10" s="26" t="inlineStr">
         <is>
           <t>Third series</t>
         </is>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="B11" s="20" t="inlineStr">
+      <c r="B11" s="26" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="C11" s="20" t="inlineStr">
+      <c r="C11" s="26" t="inlineStr">
         <is>
           <t>UI Blue Dark</t>
         </is>
       </c>
-      <c r="D11" s="20" t="inlineStr">
+      <c r="D11" s="26" t="inlineStr">
         <is>
           <t>#1344C1</t>
         </is>
       </c>
-      <c r="E11" s="24" t="inlineStr"/>
-      <c r="F11" s="20" t="inlineStr">
+      <c r="E11" s="30" t="inlineStr"/>
+      <c r="F11" s="26" t="inlineStr">
         <is>
           <t>Fourth series</t>
         </is>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="B12" s="20" t="inlineStr">
+      <c r="B12" s="26" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="C12" s="20" t="inlineStr">
+      <c r="C12" s="26" t="inlineStr">
         <is>
           <t>Indigo Light</t>
         </is>
       </c>
-      <c r="D12" s="20" t="inlineStr">
+      <c r="D12" s="26" t="inlineStr">
         <is>
           <t>#BE9DFA</t>
         </is>
       </c>
-      <c r="E12" s="25" t="inlineStr"/>
-      <c r="F12" s="20" t="inlineStr">
+      <c r="E12" s="31" t="inlineStr"/>
+      <c r="F12" s="26" t="inlineStr">
         <is>
           <t>Fifth series</t>
         </is>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="B13" s="20" t="inlineStr">
+      <c r="B13" s="26" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="C13" s="20" t="inlineStr">
+      <c r="C13" s="26" t="inlineStr">
         <is>
           <t>Dodger Dark</t>
         </is>
       </c>
-      <c r="D13" s="20" t="inlineStr">
+      <c r="D13" s="26" t="inlineStr">
         <is>
           <t>#0062A8</t>
         </is>
       </c>
-      <c r="E13" s="26" t="inlineStr"/>
-      <c r="F13" s="20" t="inlineStr">
+      <c r="E13" s="32" t="inlineStr"/>
+      <c r="F13" s="26" t="inlineStr">
         <is>
           <t>Sixth series, or fold the rest into 'Other'</t>
         </is>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="B14" s="20" t="inlineStr">
+      <c r="B14" s="26" t="inlineStr">
         <is>
           <t>Dark</t>
         </is>
       </c>
-      <c r="C14" s="20" t="inlineStr">
+      <c r="C14" s="26" t="inlineStr">
         <is>
           <t>On Tiber slides</t>
         </is>
       </c>
-      <c r="D14" s="20" t="inlineStr">
+      <c r="D14" s="26" t="inlineStr">
         <is>
           <t>#0094FF · #661DEE · #0062A8 · #9963FD</t>
         </is>
       </c>
-      <c r="E14" s="20" t="inlineStr"/>
-      <c r="F14" s="20" t="inlineStr">
+      <c r="E14" s="26" t="inlineStr"/>
+      <c r="F14" s="26" t="inlineStr">
         <is>
           <t>Four series at most on dark</t>
         </is>
@@ -3632,7 +3834,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Y14"/>
+  <dimension ref="A1:S14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.5" customWidth="1" min="1" max="1"/>
@@ -3690,12 +3892,6 @@
       <c r="Q1" s="1" t="n"/>
       <c r="R1" s="1" t="n"/>
       <c r="S1" s="1" t="n"/>
-      <c r="T1" s="1" t="n"/>
-      <c r="U1" s="1" t="n"/>
-      <c r="V1" s="1" t="n"/>
-      <c r="W1" s="1" t="n"/>
-      <c r="X1" s="1" t="n"/>
-      <c r="Y1" s="1" t="n"/>
     </row>
     <row r="2" ht="6" customHeight="1"/>
     <row r="4">
@@ -3719,123 +3915,145 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="C8" s="8">
+        <f>"  "&amp;C9&amp;"     "</f>
+        <v/>
+      </c>
+      <c r="D8" s="8">
+        <f>"  "&amp;D9&amp;"     "</f>
+        <v/>
+      </c>
+      <c r="E8" s="8">
+        <f>"  "&amp;E9&amp;"     "</f>
+        <v/>
+      </c>
+      <c r="F8" s="8">
+        <f>"  "&amp;F9&amp;"     "</f>
+        <v/>
+      </c>
+      <c r="G8" s="8">
+        <f>"  "&amp;G9&amp;"     "</f>
+        <v/>
+      </c>
+    </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="B9" s="8" t="inlineStr">
+      <c r="B9" s="9" t="inlineStr">
         <is>
           <t>Quarter</t>
         </is>
       </c>
-      <c r="C9" s="9" t="inlineStr">
+      <c r="C9" s="10" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="D9" s="9" t="inlineStr">
+      <c r="D9" s="10" t="inlineStr">
         <is>
           <t>Print</t>
         </is>
       </c>
-      <c r="E9" s="9" t="inlineStr">
+      <c r="E9" s="10" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="F9" s="9" t="inlineStr">
+      <c r="F9" s="10" t="inlineStr">
         <is>
           <t>Portal</t>
         </is>
       </c>
-      <c r="G9" s="9" t="inlineStr">
+      <c r="G9" s="10" t="inlineStr">
         <is>
           <t>App</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="10" t="inlineStr">
+      <c r="B10" s="11" t="inlineStr">
         <is>
           <t>Q1</t>
         </is>
       </c>
-      <c r="C10" s="11" t="n">
+      <c r="C10" s="12" t="n">
         <v>42000</v>
       </c>
-      <c r="D10" s="11" t="n">
+      <c r="D10" s="12" t="n">
         <v>31000</v>
       </c>
-      <c r="E10" s="11" t="n">
+      <c r="E10" s="12" t="n">
         <v>12000</v>
       </c>
-      <c r="F10" s="11" t="n">
+      <c r="F10" s="12" t="n">
         <v>21000</v>
       </c>
-      <c r="G10" s="11" t="n">
+      <c r="G10" s="12" t="n">
         <v>8000</v>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="10" t="inlineStr">
+      <c r="B11" s="11" t="inlineStr">
         <is>
           <t>Q2</t>
         </is>
       </c>
-      <c r="C11" s="11" t="n">
+      <c r="C11" s="12" t="n">
         <v>46500</v>
       </c>
-      <c r="D11" s="11" t="n">
+      <c r="D11" s="12" t="n">
         <v>29800</v>
       </c>
-      <c r="E11" s="11" t="n">
+      <c r="E11" s="12" t="n">
         <v>15400</v>
       </c>
-      <c r="F11" s="11" t="n">
+      <c r="F11" s="12" t="n">
         <v>24000</v>
       </c>
-      <c r="G11" s="11" t="n">
+      <c r="G11" s="12" t="n">
         <v>11500</v>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="10" t="inlineStr">
+      <c r="B12" s="11" t="inlineStr">
         <is>
           <t>Q3</t>
         </is>
       </c>
-      <c r="C12" s="11" t="n">
+      <c r="C12" s="12" t="n">
         <v>51200</v>
       </c>
-      <c r="D12" s="11" t="n">
+      <c r="D12" s="12" t="n">
         <v>27600</v>
       </c>
-      <c r="E12" s="11" t="n">
+      <c r="E12" s="12" t="n">
         <v>18900</v>
       </c>
-      <c r="F12" s="11" t="n">
+      <c r="F12" s="12" t="n">
         <v>26500</v>
       </c>
-      <c r="G12" s="11" t="n">
+      <c r="G12" s="12" t="n">
         <v>15800</v>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="10" t="inlineStr">
+      <c r="B13" s="11" t="inlineStr">
         <is>
           <t>Q4</t>
         </is>
       </c>
-      <c r="C13" s="11" t="n">
+      <c r="C13" s="12" t="n">
         <v>55800</v>
       </c>
-      <c r="D13" s="11" t="n">
+      <c r="D13" s="12" t="n">
         <v>26100</v>
       </c>
-      <c r="E13" s="11" t="n">
+      <c r="E13" s="12" t="n">
         <v>22300</v>
       </c>
-      <c r="F13" s="11" t="n">
+      <c r="F13" s="12" t="n">
         <v>29900</v>
       </c>
-      <c r="G13" s="11" t="n">
+      <c r="G13" s="12" t="n">
         <v>19400</v>
       </c>
     </row>
@@ -3864,7 +4082,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Y14"/>
+  <dimension ref="A1:S14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.5" customWidth="1" min="1" max="1"/>
@@ -3922,12 +4140,6 @@
       <c r="Q1" s="1" t="n"/>
       <c r="R1" s="1" t="n"/>
       <c r="S1" s="1" t="n"/>
-      <c r="T1" s="1" t="n"/>
-      <c r="U1" s="1" t="n"/>
-      <c r="V1" s="1" t="n"/>
-      <c r="W1" s="1" t="n"/>
-      <c r="X1" s="1" t="n"/>
-      <c r="Y1" s="1" t="n"/>
     </row>
     <row r="2" ht="6" customHeight="1"/>
     <row r="4">
@@ -3951,106 +4163,124 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="C8" s="8">
+        <f>"  "&amp;C9&amp;"     "</f>
+        <v/>
+      </c>
+      <c r="D8" s="8">
+        <f>"  "&amp;D9&amp;"     "</f>
+        <v/>
+      </c>
+      <c r="E8" s="8">
+        <f>"  "&amp;E9&amp;"     "</f>
+        <v/>
+      </c>
+      <c r="F8" s="8">
+        <f>"  "&amp;F9&amp;"     "</f>
+        <v/>
+      </c>
+    </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="B9" s="8" t="inlineStr">
+      <c r="B9" s="9" t="inlineStr">
         <is>
           <t>Quarter</t>
         </is>
       </c>
-      <c r="C9" s="9" t="inlineStr">
+      <c r="C9" s="10" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="D9" s="9" t="inlineStr">
+      <c r="D9" s="10" t="inlineStr">
         <is>
           <t>Print</t>
         </is>
       </c>
-      <c r="E9" s="9" t="inlineStr">
+      <c r="E9" s="10" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="F9" s="9" t="inlineStr">
+      <c r="F9" s="10" t="inlineStr">
         <is>
           <t>Portal</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="10" t="inlineStr">
+      <c r="B10" s="11" t="inlineStr">
         <is>
           <t>Q1</t>
         </is>
       </c>
-      <c r="C10" s="11" t="n">
+      <c r="C10" s="12" t="n">
         <v>42000</v>
       </c>
-      <c r="D10" s="11" t="n">
+      <c r="D10" s="12" t="n">
         <v>31000</v>
       </c>
-      <c r="E10" s="11" t="n">
+      <c r="E10" s="12" t="n">
         <v>12000</v>
       </c>
-      <c r="F10" s="11" t="n">
+      <c r="F10" s="12" t="n">
         <v>21000</v>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="10" t="inlineStr">
+      <c r="B11" s="11" t="inlineStr">
         <is>
           <t>Q2</t>
         </is>
       </c>
-      <c r="C11" s="11" t="n">
+      <c r="C11" s="12" t="n">
         <v>46500</v>
       </c>
-      <c r="D11" s="11" t="n">
+      <c r="D11" s="12" t="n">
         <v>29800</v>
       </c>
-      <c r="E11" s="11" t="n">
+      <c r="E11" s="12" t="n">
         <v>15400</v>
       </c>
-      <c r="F11" s="11" t="n">
+      <c r="F11" s="12" t="n">
         <v>24000</v>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="10" t="inlineStr">
+      <c r="B12" s="11" t="inlineStr">
         <is>
           <t>Q3</t>
         </is>
       </c>
-      <c r="C12" s="11" t="n">
+      <c r="C12" s="12" t="n">
         <v>51200</v>
       </c>
-      <c r="D12" s="11" t="n">
+      <c r="D12" s="12" t="n">
         <v>27600</v>
       </c>
-      <c r="E12" s="11" t="n">
+      <c r="E12" s="12" t="n">
         <v>18900</v>
       </c>
-      <c r="F12" s="11" t="n">
+      <c r="F12" s="12" t="n">
         <v>26500</v>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="10" t="inlineStr">
+      <c r="B13" s="11" t="inlineStr">
         <is>
           <t>Q4</t>
         </is>
       </c>
-      <c r="C13" s="11" t="n">
+      <c r="C13" s="12" t="n">
         <v>55800</v>
       </c>
-      <c r="D13" s="11" t="n">
+      <c r="D13" s="12" t="n">
         <v>26100</v>
       </c>
-      <c r="E13" s="11" t="n">
+      <c r="E13" s="12" t="n">
         <v>22300</v>
       </c>
-      <c r="F13" s="11" t="n">
+      <c r="F13" s="12" t="n">
         <v>29900</v>
       </c>
     </row>
@@ -4079,7 +4309,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Y16"/>
+  <dimension ref="A1:S16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.5" customWidth="1" min="1" max="1"/>
@@ -4137,12 +4367,6 @@
       <c r="Q1" s="1" t="n"/>
       <c r="R1" s="1" t="n"/>
       <c r="S1" s="1" t="n"/>
-      <c r="T1" s="1" t="n"/>
-      <c r="U1" s="1" t="n"/>
-      <c r="V1" s="1" t="n"/>
-      <c r="W1" s="1" t="n"/>
-      <c r="X1" s="1" t="n"/>
-      <c r="Y1" s="1" t="n"/>
     </row>
     <row r="2" ht="6" customHeight="1"/>
     <row r="4">
@@ -4167,74 +4391,74 @@
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="B9" s="8" t="inlineStr">
+      <c r="B9" s="9" t="inlineStr">
         <is>
           <t>Business unit</t>
         </is>
       </c>
-      <c r="C9" s="9" t="inlineStr">
+      <c r="C9" s="10" t="inlineStr">
         <is>
           <t>Templates</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="10" t="inlineStr">
+      <c r="B10" s="11" t="inlineStr">
         <is>
           <t>Claims</t>
         </is>
       </c>
-      <c r="C10" s="11" t="n">
+      <c r="C10" s="12" t="n">
         <v>412</v>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="10" t="inlineStr">
+      <c r="B11" s="11" t="inlineStr">
         <is>
           <t>Policy servicing</t>
         </is>
       </c>
-      <c r="C11" s="11" t="n">
+      <c r="C11" s="12" t="n">
         <v>356</v>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="10" t="inlineStr">
+      <c r="B12" s="11" t="inlineStr">
         <is>
           <t>Billing</t>
         </is>
       </c>
-      <c r="C12" s="11" t="n">
+      <c r="C12" s="12" t="n">
         <v>298</v>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="10" t="inlineStr">
+      <c r="B13" s="11" t="inlineStr">
         <is>
           <t>Onboarding</t>
         </is>
       </c>
-      <c r="C13" s="11" t="n">
+      <c r="C13" s="12" t="n">
         <v>241</v>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="10" t="inlineStr">
+      <c r="B14" s="11" t="inlineStr">
         <is>
           <t>Complaints</t>
         </is>
       </c>
-      <c r="C14" s="11" t="n">
+      <c r="C14" s="12" t="n">
         <v>167</v>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="10" t="inlineStr">
+      <c r="B15" s="11" t="inlineStr">
         <is>
           <t>Marketing</t>
         </is>
       </c>
-      <c r="C15" s="11" t="n">
+      <c r="C15" s="12" t="n">
         <v>102</v>
       </c>
     </row>
@@ -4263,7 +4487,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Y14"/>
+  <dimension ref="A1:S14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.5" customWidth="1" min="1" max="1"/>
@@ -4321,12 +4545,6 @@
       <c r="Q1" s="1" t="n"/>
       <c r="R1" s="1" t="n"/>
       <c r="S1" s="1" t="n"/>
-      <c r="T1" s="1" t="n"/>
-      <c r="U1" s="1" t="n"/>
-      <c r="V1" s="1" t="n"/>
-      <c r="W1" s="1" t="n"/>
-      <c r="X1" s="1" t="n"/>
-      <c r="Y1" s="1" t="n"/>
     </row>
     <row r="2" ht="6" customHeight="1"/>
     <row r="4">
@@ -4350,106 +4568,124 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="C8" s="8">
+        <f>"  "&amp;C9&amp;"     "</f>
+        <v/>
+      </c>
+      <c r="D8" s="8">
+        <f>"  "&amp;D9&amp;"     "</f>
+        <v/>
+      </c>
+      <c r="E8" s="8">
+        <f>"  "&amp;E9&amp;"     "</f>
+        <v/>
+      </c>
+      <c r="F8" s="8">
+        <f>"  "&amp;F9&amp;"     "</f>
+        <v/>
+      </c>
+    </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="B9" s="8" t="inlineStr">
+      <c r="B9" s="9" t="inlineStr">
         <is>
           <t>Quarter</t>
         </is>
       </c>
-      <c r="C9" s="9" t="inlineStr">
+      <c r="C9" s="10" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="D9" s="9" t="inlineStr">
+      <c r="D9" s="10" t="inlineStr">
         <is>
           <t>Portal</t>
         </is>
       </c>
-      <c r="E9" s="9" t="inlineStr">
+      <c r="E9" s="10" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="F9" s="9" t="inlineStr">
+      <c r="F9" s="10" t="inlineStr">
         <is>
           <t>Print</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="10" t="inlineStr">
+      <c r="B10" s="11" t="inlineStr">
         <is>
           <t>Q1</t>
         </is>
       </c>
-      <c r="C10" s="12" t="n">
+      <c r="C10" s="13" t="n">
         <v>38</v>
       </c>
-      <c r="D10" s="12" t="n">
+      <c r="D10" s="13" t="n">
         <v>14</v>
       </c>
-      <c r="E10" s="12" t="n">
+      <c r="E10" s="13" t="n">
         <v>11</v>
       </c>
-      <c r="F10" s="12" t="n">
+      <c r="F10" s="13" t="n">
         <v>37</v>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="10" t="inlineStr">
+      <c r="B11" s="11" t="inlineStr">
         <is>
           <t>Q2</t>
         </is>
       </c>
-      <c r="C11" s="12" t="n">
+      <c r="C11" s="13" t="n">
         <v>41</v>
       </c>
-      <c r="D11" s="12" t="n">
+      <c r="D11" s="13" t="n">
         <v>17</v>
       </c>
-      <c r="E11" s="12" t="n">
+      <c r="E11" s="13" t="n">
         <v>13</v>
       </c>
-      <c r="F11" s="12" t="n">
+      <c r="F11" s="13" t="n">
         <v>29</v>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="10" t="inlineStr">
+      <c r="B12" s="11" t="inlineStr">
         <is>
           <t>Q3</t>
         </is>
       </c>
-      <c r="C12" s="12" t="n">
+      <c r="C12" s="13" t="n">
         <v>44</v>
       </c>
-      <c r="D12" s="12" t="n">
+      <c r="D12" s="13" t="n">
         <v>19</v>
       </c>
-      <c r="E12" s="12" t="n">
+      <c r="E12" s="13" t="n">
         <v>14</v>
       </c>
-      <c r="F12" s="12" t="n">
+      <c r="F12" s="13" t="n">
         <v>23</v>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="10" t="inlineStr">
+      <c r="B13" s="11" t="inlineStr">
         <is>
           <t>Q4</t>
         </is>
       </c>
-      <c r="C13" s="12" t="n">
+      <c r="C13" s="13" t="n">
         <v>46</v>
       </c>
-      <c r="D13" s="12" t="n">
+      <c r="D13" s="13" t="n">
         <v>22</v>
       </c>
-      <c r="E13" s="12" t="n">
+      <c r="E13" s="13" t="n">
         <v>16</v>
       </c>
-      <c r="F13" s="12" t="n">
+      <c r="F13" s="13" t="n">
         <v>16</v>
       </c>
     </row>
@@ -4478,7 +4714,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Y22"/>
+  <dimension ref="A1:S22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.5" customWidth="1" min="1" max="1"/>
@@ -4536,12 +4772,6 @@
       <c r="Q1" s="1" t="n"/>
       <c r="R1" s="1" t="n"/>
       <c r="S1" s="1" t="n"/>
-      <c r="T1" s="1" t="n"/>
-      <c r="U1" s="1" t="n"/>
-      <c r="V1" s="1" t="n"/>
-      <c r="W1" s="1" t="n"/>
-      <c r="X1" s="1" t="n"/>
-      <c r="Y1" s="1" t="n"/>
     </row>
     <row r="2" ht="6" customHeight="1"/>
     <row r="4">
@@ -4565,176 +4795,186 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="C8" s="8">
+        <f>"  "&amp;C9&amp;"     "</f>
+        <v/>
+      </c>
+      <c r="D8" s="8">
+        <f>"  "&amp;D9&amp;"     "</f>
+        <v/>
+      </c>
+    </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="B9" s="8" t="inlineStr">
+      <c r="B9" s="9" t="inlineStr">
         <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="C9" s="9" t="inlineStr">
+      <c r="C9" s="10" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="D9" s="9" t="inlineStr">
+      <c r="D9" s="10" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="10" t="inlineStr">
+      <c r="B10" s="11" t="inlineStr">
         <is>
           <t>Jan</t>
         </is>
       </c>
-      <c r="C10" s="11" t="n">
+      <c r="C10" s="12" t="n">
         <v>21</v>
       </c>
-      <c r="D10" s="11" t="n">
+      <c r="D10" s="12" t="n">
         <v>24</v>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="10" t="inlineStr">
+      <c r="B11" s="11" t="inlineStr">
         <is>
           <t>Feb</t>
         </is>
       </c>
-      <c r="C11" s="11" t="n">
+      <c r="C11" s="12" t="n">
         <v>19</v>
       </c>
-      <c r="D11" s="11" t="n">
+      <c r="D11" s="12" t="n">
         <v>24</v>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="10" t="inlineStr">
+      <c r="B12" s="11" t="inlineStr">
         <is>
           <t>Mar</t>
         </is>
       </c>
-      <c r="C12" s="11" t="n">
+      <c r="C12" s="12" t="n">
         <v>18</v>
       </c>
-      <c r="D12" s="11" t="n">
+      <c r="D12" s="12" t="n">
         <v>23</v>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="10" t="inlineStr">
+      <c r="B13" s="11" t="inlineStr">
         <is>
           <t>Apr</t>
         </is>
       </c>
-      <c r="C13" s="11" t="n">
+      <c r="C13" s="12" t="n">
         <v>16</v>
       </c>
-      <c r="D13" s="11" t="n">
+      <c r="D13" s="12" t="n">
         <v>23</v>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="10" t="inlineStr">
+      <c r="B14" s="11" t="inlineStr">
         <is>
           <t>May</t>
         </is>
       </c>
-      <c r="C14" s="11" t="n">
+      <c r="C14" s="12" t="n">
         <v>15</v>
       </c>
-      <c r="D14" s="11" t="n">
+      <c r="D14" s="12" t="n">
         <v>22</v>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="10" t="inlineStr">
+      <c r="B15" s="11" t="inlineStr">
         <is>
           <t>Jun</t>
         </is>
       </c>
-      <c r="C15" s="11" t="n">
+      <c r="C15" s="12" t="n">
         <v>13</v>
       </c>
-      <c r="D15" s="11" t="n">
+      <c r="D15" s="12" t="n">
         <v>22</v>
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="10" t="inlineStr">
+      <c r="B16" s="11" t="inlineStr">
         <is>
           <t>Jul</t>
         </is>
       </c>
-      <c r="C16" s="11" t="n">
+      <c r="C16" s="12" t="n">
         <v>12</v>
       </c>
-      <c r="D16" s="11" t="n">
+      <c r="D16" s="12" t="n">
         <v>21</v>
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="10" t="inlineStr">
+      <c r="B17" s="11" t="inlineStr">
         <is>
           <t>Aug</t>
         </is>
       </c>
-      <c r="C17" s="11" t="n">
+      <c r="C17" s="12" t="n">
         <v>11</v>
       </c>
-      <c r="D17" s="11" t="n">
+      <c r="D17" s="12" t="n">
         <v>21</v>
       </c>
     </row>
     <row r="18">
-      <c r="B18" s="10" t="inlineStr">
+      <c r="B18" s="11" t="inlineStr">
         <is>
           <t>Sep</t>
         </is>
       </c>
-      <c r="C18" s="11" t="n">
+      <c r="C18" s="12" t="n">
         <v>10</v>
       </c>
-      <c r="D18" s="11" t="n">
+      <c r="D18" s="12" t="n">
         <v>21</v>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="10" t="inlineStr">
+      <c r="B19" s="11" t="inlineStr">
         <is>
           <t>Oct</t>
         </is>
       </c>
-      <c r="C19" s="11" t="n">
+      <c r="C19" s="12" t="n">
         <v>9</v>
       </c>
-      <c r="D19" s="11" t="n">
+      <c r="D19" s="12" t="n">
         <v>20</v>
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="10" t="inlineStr">
+      <c r="B20" s="11" t="inlineStr">
         <is>
           <t>Nov</t>
         </is>
       </c>
-      <c r="C20" s="11" t="n">
+      <c r="C20" s="12" t="n">
         <v>8</v>
       </c>
-      <c r="D20" s="11" t="n">
+      <c r="D20" s="12" t="n">
         <v>20</v>
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="10" t="inlineStr">
+      <c r="B21" s="11" t="inlineStr">
         <is>
           <t>Dec</t>
         </is>
       </c>
-      <c r="C21" s="11" t="n">
+      <c r="C21" s="12" t="n">
         <v>7</v>
       </c>
-      <c r="D21" s="11" t="n">
+      <c r="D21" s="12" t="n">
         <v>20</v>
       </c>
     </row>
@@ -4763,7 +5003,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Y16"/>
+  <dimension ref="A1:S16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.5" customWidth="1" min="1" max="1"/>
@@ -4821,12 +5061,6 @@
       <c r="Q1" s="1" t="n"/>
       <c r="R1" s="1" t="n"/>
       <c r="S1" s="1" t="n"/>
-      <c r="T1" s="1" t="n"/>
-      <c r="U1" s="1" t="n"/>
-      <c r="V1" s="1" t="n"/>
-      <c r="W1" s="1" t="n"/>
-      <c r="X1" s="1" t="n"/>
-      <c r="Y1" s="1" t="n"/>
     </row>
     <row r="2" ht="6" customHeight="1"/>
     <row r="4">
@@ -4850,126 +5084,136 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="C8" s="8">
+        <f>"  "&amp;C9&amp;"     "</f>
+        <v/>
+      </c>
+      <c r="D8" s="8">
+        <f>"  "&amp;D9&amp;"     "</f>
+        <v/>
+      </c>
+    </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="B9" s="8" t="inlineStr">
+      <c r="B9" s="9" t="inlineStr">
         <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="C9" s="9" t="inlineStr">
+      <c r="C9" s="10" t="inlineStr">
         <is>
           <t>Migrated</t>
         </is>
       </c>
-      <c r="D9" s="9" t="inlineStr">
+      <c r="D9" s="10" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="E9" s="9" t="inlineStr">
+      <c r="E9" s="10" t="inlineStr">
         <is>
           <t>vs. target</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="10" t="inlineStr">
+      <c r="B10" s="11" t="inlineStr">
         <is>
           <t>Jan</t>
         </is>
       </c>
-      <c r="C10" s="11" t="n">
+      <c r="C10" s="12" t="n">
         <v>182</v>
       </c>
-      <c r="D10" s="11" t="n">
+      <c r="D10" s="12" t="n">
         <v>200</v>
       </c>
-      <c r="E10" s="13">
+      <c r="E10" s="14">
         <f>IF(D10=0,0,C10/D10-1)</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="10" t="inlineStr">
+      <c r="B11" s="11" t="inlineStr">
         <is>
           <t>Feb</t>
         </is>
       </c>
-      <c r="C11" s="11" t="n">
+      <c r="C11" s="12" t="n">
         <v>196</v>
       </c>
-      <c r="D11" s="11" t="n">
+      <c r="D11" s="12" t="n">
         <v>210</v>
       </c>
-      <c r="E11" s="13">
+      <c r="E11" s="14">
         <f>IF(D11=0,0,C11/D11-1)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="10" t="inlineStr">
+      <c r="B12" s="11" t="inlineStr">
         <is>
           <t>Mar</t>
         </is>
       </c>
-      <c r="C12" s="11" t="n">
+      <c r="C12" s="12" t="n">
         <v>228</v>
       </c>
-      <c r="D12" s="11" t="n">
+      <c r="D12" s="12" t="n">
         <v>220</v>
       </c>
-      <c r="E12" s="13">
+      <c r="E12" s="14">
         <f>IF(D12=0,0,C12/D12-1)</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="10" t="inlineStr">
+      <c r="B13" s="11" t="inlineStr">
         <is>
           <t>Apr</t>
         </is>
       </c>
-      <c r="C13" s="11" t="n">
+      <c r="C13" s="12" t="n">
         <v>241</v>
       </c>
-      <c r="D13" s="11" t="n">
+      <c r="D13" s="12" t="n">
         <v>235</v>
       </c>
-      <c r="E13" s="13">
+      <c r="E13" s="14">
         <f>IF(D13=0,0,C13/D13-1)</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="10" t="inlineStr">
+      <c r="B14" s="11" t="inlineStr">
         <is>
           <t>May</t>
         </is>
       </c>
-      <c r="C14" s="11" t="n">
+      <c r="C14" s="12" t="n">
         <v>263</v>
       </c>
-      <c r="D14" s="11" t="n">
+      <c r="D14" s="12" t="n">
         <v>250</v>
       </c>
-      <c r="E14" s="13">
+      <c r="E14" s="14">
         <f>IF(D14=0,0,C14/D14-1)</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="10" t="inlineStr">
+      <c r="B15" s="11" t="inlineStr">
         <is>
           <t>Jun</t>
         </is>
       </c>
-      <c r="C15" s="11" t="n">
+      <c r="C15" s="12" t="n">
         <v>288</v>
       </c>
-      <c r="D15" s="11" t="n">
+      <c r="D15" s="12" t="n">
         <v>265</v>
       </c>
-      <c r="E15" s="13">
+      <c r="E15" s="14">
         <f>IF(D15=0,0,C15/D15-1)</f>
         <v/>
       </c>
@@ -4999,7 +5243,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Y16"/>
+  <dimension ref="A1:S16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.5" customWidth="1" min="1" max="1"/>
@@ -5057,12 +5301,6 @@
       <c r="Q1" s="1" t="n"/>
       <c r="R1" s="1" t="n"/>
       <c r="S1" s="1" t="n"/>
-      <c r="T1" s="1" t="n"/>
-      <c r="U1" s="1" t="n"/>
-      <c r="V1" s="1" t="n"/>
-      <c r="W1" s="1" t="n"/>
-      <c r="X1" s="1" t="n"/>
-      <c r="Y1" s="1" t="n"/>
     </row>
     <row r="2" ht="6" customHeight="1"/>
     <row r="4">
@@ -5087,74 +5325,74 @@
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="B9" s="8" t="inlineStr">
+      <c r="B9" s="9" t="inlineStr">
         <is>
           <t>Channel</t>
         </is>
       </c>
-      <c r="C9" s="9" t="inlineStr">
+      <c r="C9" s="10" t="inlineStr">
         <is>
           <t>Share</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="10" t="inlineStr">
+      <c r="B10" s="11" t="inlineStr">
         <is>
           <t>Web portal</t>
         </is>
       </c>
-      <c r="C10" s="14" t="n">
+      <c r="C10" s="15" t="n">
         <v>0.38</v>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="10" t="inlineStr">
+      <c r="B11" s="11" t="inlineStr">
         <is>
           <t>Mobile app</t>
         </is>
       </c>
-      <c r="C11" s="14" t="n">
+      <c r="C11" s="15" t="n">
         <v>0.24</v>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="10" t="inlineStr">
+      <c r="B12" s="11" t="inlineStr">
         <is>
           <t>Agent-assisted</t>
         </is>
       </c>
-      <c r="C12" s="14" t="n">
+      <c r="C12" s="15" t="n">
         <v>0.17</v>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="10" t="inlineStr">
+      <c r="B13" s="11" t="inlineStr">
         <is>
           <t>Email link</t>
         </is>
       </c>
-      <c r="C13" s="14" t="n">
+      <c r="C13" s="15" t="n">
         <v>0.13</v>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="10" t="inlineStr">
+      <c r="B14" s="11" t="inlineStr">
         <is>
           <t>Paper form</t>
         </is>
       </c>
-      <c r="C14" s="14" t="n">
+      <c r="C14" s="15" t="n">
         <v>0.08</v>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="15" t="inlineStr">
+      <c r="B15" s="16" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="C15" s="16">
+      <c r="C15" s="17">
         <f>SUM(C10:C14)</f>
         <v/>
       </c>
@@ -5184,7 +5422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Y12"/>
+  <dimension ref="A1:S12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.5" customWidth="1" min="1" max="1"/>
@@ -5192,9 +5430,9 @@
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="3" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
@@ -5222,7 +5460,7 @@
       <c r="A1" s="1" t="n"/>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>Table · KPIs with data bars</t>
+          <t>Table · KPIs with progress bars</t>
         </is>
       </c>
       <c r="C1" s="1" t="n"/>
@@ -5242,12 +5480,6 @@
       <c r="Q1" s="1" t="n"/>
       <c r="R1" s="1" t="n"/>
       <c r="S1" s="1" t="n"/>
-      <c r="T1" s="1" t="n"/>
-      <c r="U1" s="1" t="n"/>
-      <c r="V1" s="1" t="n"/>
-      <c r="W1" s="1" t="n"/>
-      <c r="X1" s="1" t="n"/>
-      <c r="Y1" s="1" t="n"/>
     </row>
     <row r="2" ht="6" customHeight="1"/>
     <row r="4">
@@ -5258,136 +5490,186 @@
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="9" t="inlineStr">
         <is>
           <t>Program</t>
         </is>
       </c>
-      <c r="C7" s="9" t="inlineStr">
+      <c r="C7" s="10" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="D7" s="9" t="inlineStr">
+      <c r="D7" s="10" t="inlineStr">
         <is>
           <t>Actual</t>
         </is>
       </c>
-      <c r="E7" s="9" t="inlineStr">
+      <c r="E7" s="10" t="inlineStr">
         <is>
           <t>vs. target</t>
         </is>
       </c>
-      <c r="F7" s="9" t="inlineStr">
+      <c r="F7" s="10" t="inlineStr"/>
+      <c r="G7" s="9" t="inlineStr">
         <is>
           <t>Progress</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="B8" s="10" t="inlineStr">
+    <row r="8" ht="24" customHeight="1">
+      <c r="B8" s="18" t="inlineStr">
         <is>
           <t>Template consolidation</t>
         </is>
       </c>
-      <c r="C8" s="11" t="n">
+      <c r="C8" s="19" t="n">
         <v>1200</v>
       </c>
-      <c r="D8" s="11" t="n">
+      <c r="D8" s="19" t="n">
         <v>1056</v>
       </c>
-      <c r="E8" s="13">
+      <c r="E8" s="20">
         <f>IF(C8=0,0,D8/C8-1)</f>
         <v/>
       </c>
-      <c r="F8" s="17">
+      <c r="F8" s="21" t="n"/>
+      <c r="G8" s="22">
         <f>IF(C8=0,0,MIN(1,D8/C8))</f>
         <v/>
       </c>
-    </row>
-    <row r="9">
-      <c r="B9" s="10" t="inlineStr">
+      <c r="H8" s="23">
+        <f>G8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" ht="24" customHeight="1">
+      <c r="B9" s="18" t="inlineStr">
         <is>
           <t>Digital adoption</t>
         </is>
       </c>
-      <c r="C9" s="18" t="n">
+      <c r="C9" s="24" t="n">
         <v>0.6</v>
       </c>
-      <c r="D9" s="18" t="n">
+      <c r="D9" s="24" t="n">
         <v>0.54</v>
       </c>
-      <c r="E9" s="13">
+      <c r="E9" s="20">
         <f>IF(C9=0,0,D9/C9-1)</f>
         <v/>
       </c>
-      <c r="F9" s="17">
+      <c r="F9" s="21" t="n"/>
+      <c r="G9" s="22">
         <f>IF(C9=0,0,MIN(1,D9/C9))</f>
         <v/>
       </c>
-    </row>
-    <row r="10">
-      <c r="B10" s="10" t="inlineStr">
+      <c r="H9" s="23">
+        <f>G9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="24" customHeight="1">
+      <c r="B10" s="18" t="inlineStr">
         <is>
           <t>Straight-through processing</t>
         </is>
       </c>
-      <c r="C10" s="18" t="n">
+      <c r="C10" s="24" t="n">
         <v>0.85</v>
       </c>
-      <c r="D10" s="18" t="n">
+      <c r="D10" s="24" t="n">
         <v>0.8100000000000001</v>
       </c>
-      <c r="E10" s="13">
+      <c r="E10" s="20">
         <f>IF(C10=0,0,D10/C10-1)</f>
         <v/>
       </c>
-      <c r="F10" s="17">
+      <c r="F10" s="21" t="n"/>
+      <c r="G10" s="22">
         <f>IF(C10=0,0,MIN(1,D10/C10))</f>
         <v/>
       </c>
-    </row>
-    <row r="11">
-      <c r="B11" s="10" t="inlineStr">
+      <c r="H10" s="23">
+        <f>G10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="24" customHeight="1">
+      <c r="B11" s="18" t="inlineStr">
         <is>
           <t>Self-service forms live</t>
         </is>
       </c>
-      <c r="C11" s="11" t="n">
+      <c r="C11" s="19" t="n">
         <v>40</v>
       </c>
-      <c r="D11" s="11" t="n">
+      <c r="D11" s="19" t="n">
         <v>46</v>
       </c>
-      <c r="E11" s="13">
+      <c r="E11" s="20">
         <f>IF(C11=0,0,D11/C11-1)</f>
         <v/>
       </c>
-      <c r="F11" s="17">
+      <c r="F11" s="21" t="n"/>
+      <c r="G11" s="22">
         <f>IF(C11=0,0,MIN(1,D11/C11))</f>
         <v/>
       </c>
+      <c r="H11" s="23">
+        <f>G11</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>Sample data is illustrative. Replace it with your own and cite the source under the table. 'vs. target' and 'Progress' are formulas.</t>
+          <t>Sample data is illustrative. Replace it with your own and cite the source under the table. 'vs. target' and 'Progress' are formulas; bars stop at 100%.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="F8:F11">
+  <mergeCells count="1">
+    <mergeCell ref="G7:H7"/>
+  </mergeCells>
+  <conditionalFormatting sqref="H8:H11">
     <cfRule type="dataBar" priority="1">
-      <dataBar showValue="1">
+      <dataBar minLength="0" maxLength="100" showValue="0">
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="1"/>
         <color rgb="000094FF"/>
       </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{5C1F0B2A-7D3E-4C59-9A61-0094FF2026AA}</x14:id>
+        </ext>
+      </extLst>
     </cfRule>
   </conditionalFormatting>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="1" fitToWidth="1"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
+      <x14:conditionalFormattings>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{5C1F0B2A-7D3E-4C59-9A61-0094FF2026AA}">
+            <x14:dataBar minLength="0" maxLength="100" gradient="0" border="0">
+              <x14:cfvo type="num">
+                <xm:f>0</xm:f>
+              </x14:cfvo>
+              <x14:cfvo type="num">
+                <xm:f>1</xm:f>
+              </x14:cfvo>
+              <x14:negativeFillColor rgb="FF661DEE"/>
+              <x14:axisColor rgb="FF677C91"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>H8:H11</xm:sqref>
+        </x14:conditionalFormatting>
+      </x14:conditionalFormattings>
+    </ext>
+  </extLst>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Excel templates: title left with key right, tighter keys, centered doughnut
Chart titles sit on the left with the key on the right of the same band; keys wrap to
a second row when they don't fit, with less space between entries. The Bar chart gets
more room under its title. The doughnut is centered under its title with its key to
the right, padded key names to match the other charts, a 'Key' heading aligned to the
squares, and thinner slice outlines so the ring stays a true circle.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/site/assets/downloads/SmartCommunications_Excel_Chart_Templates.xlsx
+++ b/site/assets/downloads/SmartCommunications_Excel_Chart_Templates.xlsx
@@ -324,7 +324,7 @@
           <strCache>
             <ptCount val="1"/>
             <pt idx="0">
-              <v>Communications sent by channel</v>
+              <v>Communications by channel</v>
             </pt>
           </strCache>
         </strRef>
@@ -364,6 +364,18 @@
       </txPr>
     </title>
     <plotArea>
+      <layout>
+        <manualLayout>
+          <xMode val="edge"/>
+          <yMode val="edge"/>
+          <wMode val="factor"/>
+          <hMode val="factor"/>
+          <x val="0.02"/>
+          <y val="0.225"/>
+          <w val="0.96"/>
+          <h val="0.7050000000000001"/>
+        </manualLayout>
+      </layout>
       <barChart>
         <barDir val="col"/>
         <grouping val="clustered"/>
@@ -376,7 +388,7 @@
               <strCache>
                 <ptCount val="1"/>
                 <pt idx="0">
-                  <v xml:space="preserve">  Email     </v>
+                  <v xml:space="preserve"> Email  </v>
                 </pt>
               </strCache>
             </strRef>
@@ -410,7 +422,7 @@
               <strCache>
                 <ptCount val="1"/>
                 <pt idx="0">
-                  <v xml:space="preserve">  Print     </v>
+                  <v xml:space="preserve"> Print  </v>
                 </pt>
               </strCache>
             </strRef>
@@ -444,7 +456,7 @@
               <strCache>
                 <ptCount val="1"/>
                 <pt idx="0">
-                  <v xml:space="preserve">  SMS     </v>
+                  <v xml:space="preserve"> SMS  </v>
                 </pt>
               </strCache>
             </strRef>
@@ -478,7 +490,7 @@
               <strCache>
                 <ptCount val="1"/>
                 <pt idx="0">
-                  <v xml:space="preserve">  Portal     </v>
+                  <v xml:space="preserve"> Portal  </v>
                 </pt>
               </strCache>
             </strRef>
@@ -512,7 +524,7 @@
               <strCache>
                 <ptCount val="1"/>
                 <pt idx="0">
-                  <v xml:space="preserve">  App     </v>
+                  <v xml:space="preserve"> App  </v>
                 </pt>
               </strCache>
             </strRef>
@@ -644,12 +656,24 @@
     </plotArea>
     <legend>
       <legendPos val="t"/>
+      <layout>
+        <manualLayout>
+          <xMode val="edge"/>
+          <yMode val="edge"/>
+          <wMode val="factor"/>
+          <hMode val="factor"/>
+          <x val="0.4831647727272727"/>
+          <y val="0.035"/>
+          <w val="0.4968352272727273"/>
+          <h val="0.14"/>
+        </manualLayout>
+      </layout>
       <overlay val="0"/>
       <txPr>
         <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
         <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
-            <a:defRPr sz="1400" b="0">
+            <a:defRPr sz="1500" b="0">
               <a:solidFill>
                 <a:srgbClr val="183958"/>
               </a:solidFill>
@@ -659,7 +683,7 @@
           <a:r>
             <a:t/>
           </a:r>
-          <a:endParaRPr sz="1400" b="0">
+          <a:endParaRPr sz="1500" b="0">
             <a:solidFill>
               <a:srgbClr val="183958"/>
             </a:solidFill>
@@ -694,7 +718,7 @@
           <strCache>
             <ptCount val="1"/>
             <pt idx="0">
-              <v>Communications sent by channel</v>
+              <v>Communications by channel</v>
             </pt>
           </strCache>
         </strRef>
@@ -734,6 +758,18 @@
       </txPr>
     </title>
     <plotArea>
+      <layout>
+        <manualLayout>
+          <xMode val="edge"/>
+          <yMode val="edge"/>
+          <wMode val="factor"/>
+          <hMode val="factor"/>
+          <x val="0.02"/>
+          <y val="0.16"/>
+          <w val="0.96"/>
+          <h val="0.77"/>
+        </manualLayout>
+      </layout>
       <barChart>
         <barDir val="col"/>
         <grouping val="clustered"/>
@@ -746,7 +782,7 @@
               <strCache>
                 <ptCount val="1"/>
                 <pt idx="0">
-                  <v xml:space="preserve">  Email     </v>
+                  <v xml:space="preserve"> Email  </v>
                 </pt>
               </strCache>
             </strRef>
@@ -780,7 +816,7 @@
               <strCache>
                 <ptCount val="1"/>
                 <pt idx="0">
-                  <v xml:space="preserve">  Print     </v>
+                  <v xml:space="preserve"> Print  </v>
                 </pt>
               </strCache>
             </strRef>
@@ -814,7 +850,7 @@
               <strCache>
                 <ptCount val="1"/>
                 <pt idx="0">
-                  <v xml:space="preserve">  SMS     </v>
+                  <v xml:space="preserve"> SMS  </v>
                 </pt>
               </strCache>
             </strRef>
@@ -848,7 +884,7 @@
               <strCache>
                 <ptCount val="1"/>
                 <pt idx="0">
-                  <v xml:space="preserve">  Portal     </v>
+                  <v xml:space="preserve"> Portal  </v>
                 </pt>
               </strCache>
             </strRef>
@@ -980,12 +1016,24 @@
     </plotArea>
     <legend>
       <legendPos val="t"/>
+      <layout>
+        <manualLayout>
+          <xMode val="edge"/>
+          <yMode val="edge"/>
+          <wMode val="factor"/>
+          <hMode val="factor"/>
+          <x val="0.5110530081084281"/>
+          <y val="0.035"/>
+          <w val="0.4689469918915719"/>
+          <h val="0.075"/>
+        </manualLayout>
+      </layout>
       <overlay val="0"/>
       <txPr>
         <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
         <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
-            <a:defRPr sz="1400" b="0">
+            <a:defRPr sz="1500" b="0">
               <a:solidFill>
                 <a:srgbClr val="FFFFFF"/>
               </a:solidFill>
@@ -995,7 +1043,7 @@
           <a:r>
             <a:t/>
           </a:r>
-          <a:endParaRPr sz="1400" b="0">
+          <a:endParaRPr sz="1500" b="0">
             <a:solidFill>
               <a:srgbClr val="FFFFFF"/>
             </a:solidFill>
@@ -1070,6 +1118,18 @@
       </txPr>
     </title>
     <plotArea>
+      <layout>
+        <manualLayout>
+          <xMode val="edge"/>
+          <yMode val="edge"/>
+          <wMode val="factor"/>
+          <hMode val="factor"/>
+          <x val="0.02"/>
+          <y val="0.17"/>
+          <w val="0.93"/>
+          <h val="0.8"/>
+        </manualLayout>
+      </layout>
       <barChart>
         <barDir val="bar"/>
         <grouping val="clustered"/>
@@ -1292,6 +1352,18 @@
       </txPr>
     </title>
     <plotArea>
+      <layout>
+        <manualLayout>
+          <xMode val="edge"/>
+          <yMode val="edge"/>
+          <wMode val="factor"/>
+          <hMode val="factor"/>
+          <x val="0.02"/>
+          <y val="0.16"/>
+          <w val="0.96"/>
+          <h val="0.77"/>
+        </manualLayout>
+      </layout>
       <barChart>
         <barDir val="col"/>
         <grouping val="percentStacked"/>
@@ -1304,7 +1376,7 @@
               <strCache>
                 <ptCount val="1"/>
                 <pt idx="0">
-                  <v xml:space="preserve">  Email     </v>
+                  <v xml:space="preserve"> Email   </v>
                 </pt>
               </strCache>
             </strRef>
@@ -1340,7 +1412,7 @@
               <strCache>
                 <ptCount val="1"/>
                 <pt idx="0">
-                  <v xml:space="preserve">  Portal     </v>
+                  <v xml:space="preserve"> Portal   </v>
                 </pt>
               </strCache>
             </strRef>
@@ -1376,7 +1448,7 @@
               <strCache>
                 <ptCount val="1"/>
                 <pt idx="0">
-                  <v xml:space="preserve">  SMS     </v>
+                  <v xml:space="preserve"> SMS   </v>
                 </pt>
               </strCache>
             </strRef>
@@ -1412,7 +1484,7 @@
               <strCache>
                 <ptCount val="1"/>
                 <pt idx="0">
-                  <v xml:space="preserve">  Print     </v>
+                  <v xml:space="preserve"> Print   </v>
                 </pt>
               </strCache>
             </strRef>
@@ -1546,12 +1618,24 @@
     </plotArea>
     <legend>
       <legendPos val="t"/>
+      <layout>
+        <manualLayout>
+          <xMode val="edge"/>
+          <yMode val="edge"/>
+          <wMode val="factor"/>
+          <hMode val="factor"/>
+          <x val="0.4845946747750948"/>
+          <y val="0.035"/>
+          <w val="0.4954053252249052"/>
+          <h val="0.075"/>
+        </manualLayout>
+      </layout>
       <overlay val="0"/>
       <txPr>
         <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
         <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
-            <a:defRPr sz="1400" b="0">
+            <a:defRPr sz="1500" b="0">
               <a:solidFill>
                 <a:srgbClr val="183958"/>
               </a:solidFill>
@@ -1561,7 +1645,7 @@
           <a:r>
             <a:t/>
           </a:r>
-          <a:endParaRPr sz="1400" b="0">
+          <a:endParaRPr sz="1500" b="0">
             <a:solidFill>
               <a:srgbClr val="183958"/>
             </a:solidFill>
@@ -1636,6 +1720,18 @@
       </txPr>
     </title>
     <plotArea>
+      <layout>
+        <manualLayout>
+          <xMode val="edge"/>
+          <yMode val="edge"/>
+          <wMode val="factor"/>
+          <hMode val="factor"/>
+          <x val="0.02"/>
+          <y val="0.16"/>
+          <w val="0.96"/>
+          <h val="0.77"/>
+        </manualLayout>
+      </layout>
       <lineChart>
         <grouping val="standard"/>
         <ser>
@@ -1647,7 +1743,7 @@
               <strCache>
                 <ptCount val="1"/>
                 <pt idx="0">
-                  <v xml:space="preserve">  2026     </v>
+                  <v xml:space="preserve"> 2026   </v>
                 </pt>
               </strCache>
             </strRef>
@@ -1689,7 +1785,7 @@
               <strCache>
                 <ptCount val="1"/>
                 <pt idx="0">
-                  <v xml:space="preserve">  2025     </v>
+                  <v xml:space="preserve"> 2025   </v>
                 </pt>
               </strCache>
             </strRef>
@@ -1827,12 +1923,24 @@
     </plotArea>
     <legend>
       <legendPos val="t"/>
+      <layout>
+        <manualLayout>
+          <xMode val="edge"/>
+          <yMode val="edge"/>
+          <wMode val="factor"/>
+          <hMode val="factor"/>
+          <x val="0.6396136363636363"/>
+          <y val="0.035"/>
+          <w val="0.3403863636363637"/>
+          <h val="0.075"/>
+        </manualLayout>
+      </layout>
       <overlay val="0"/>
       <txPr>
         <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
         <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
-            <a:defRPr sz="1400" b="0">
+            <a:defRPr sz="1500" b="0">
               <a:solidFill>
                 <a:srgbClr val="183958"/>
               </a:solidFill>
@@ -1842,7 +1950,7 @@
           <a:r>
             <a:t/>
           </a:r>
-          <a:endParaRPr sz="1400" b="0">
+          <a:endParaRPr sz="1500" b="0">
             <a:solidFill>
               <a:srgbClr val="183958"/>
             </a:solidFill>
@@ -1917,6 +2025,18 @@
       </txPr>
     </title>
     <plotArea>
+      <layout>
+        <manualLayout>
+          <xMode val="edge"/>
+          <yMode val="edge"/>
+          <wMode val="factor"/>
+          <hMode val="factor"/>
+          <x val="0.02"/>
+          <y val="0.16"/>
+          <w val="0.96"/>
+          <h val="0.77"/>
+        </manualLayout>
+      </layout>
       <barChart>
         <barDir val="col"/>
         <grouping val="clustered"/>
@@ -1929,7 +2049,7 @@
               <strCache>
                 <ptCount val="1"/>
                 <pt idx="0">
-                  <v xml:space="preserve">  Migrated     </v>
+                  <v xml:space="preserve"> Migrated   </v>
                 </pt>
               </strCache>
             </strRef>
@@ -1969,7 +2089,7 @@
               <strCache>
                 <ptCount val="1"/>
                 <pt idx="0">
-                  <v xml:space="preserve">  Target     </v>
+                  <v xml:space="preserve"> Target   </v>
                 </pt>
               </strCache>
             </strRef>
@@ -2108,12 +2228,24 @@
     </plotArea>
     <legend>
       <legendPos val="t"/>
+      <layout>
+        <manualLayout>
+          <xMode val="edge"/>
+          <yMode val="edge"/>
+          <wMode val="factor"/>
+          <hMode val="factor"/>
+          <x val="0.6215005770596591"/>
+          <y val="0.035"/>
+          <w val="0.3584994229403409"/>
+          <h val="0.075"/>
+        </manualLayout>
+      </layout>
       <overlay val="0"/>
       <txPr>
         <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
         <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
-            <a:defRPr sz="1400" b="0">
+            <a:defRPr sz="1500" b="0">
               <a:solidFill>
                 <a:srgbClr val="183958"/>
               </a:solidFill>
@@ -2123,7 +2255,7 @@
           <a:r>
             <a:t/>
           </a:r>
-          <a:endParaRPr sz="1400" b="0">
+          <a:endParaRPr sz="1500" b="0">
             <a:solidFill>
               <a:srgbClr val="183958"/>
             </a:solidFill>
@@ -2163,16 +2295,6 @@
           </strCache>
         </strRef>
       </tx>
-      <layout>
-        <manualLayout>
-          <xMode val="edge"/>
-          <yMode val="edge"/>
-          <wMode val="factor"/>
-          <hMode val="factor"/>
-          <x val="0.02"/>
-          <y val="0.03"/>
-        </manualLayout>
-      </layout>
       <overlay val="0"/>
       <txPr>
         <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
@@ -2204,10 +2326,10 @@
           <yMode val="edge"/>
           <wMode val="factor"/>
           <hMode val="factor"/>
-          <x val="0.04"/>
-          <y val="0.17"/>
-          <w val="0.52"/>
-          <h val="0.78"/>
+          <x val="0.2858181818181819"/>
+          <y val="0.19"/>
+          <w val="0.4283636363636363"/>
+          <h val="0.76"/>
         </manualLayout>
       </layout>
       <doughnutChart>
@@ -2231,7 +2353,7 @@
               <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="0094FF"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
                 <a:solidFill>
                   <a:srgbClr val="FFFFFF"/>
                 </a:solidFill>
@@ -2245,7 +2367,7 @@
               <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="661DEE"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
                 <a:solidFill>
                   <a:srgbClr val="FFFFFF"/>
                 </a:solidFill>
@@ -2259,7 +2381,7 @@
               <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="57B8FF"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
                 <a:solidFill>
                   <a:srgbClr val="FFFFFF"/>
                 </a:solidFill>
@@ -2273,7 +2395,7 @@
               <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="1344C1"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
                 <a:solidFill>
                   <a:srgbClr val="FFFFFF"/>
                 </a:solidFill>
@@ -2287,7 +2409,7 @@
               <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="BE9DFA"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
                 <a:solidFill>
                   <a:srgbClr val="FFFFFF"/>
                 </a:solidFill>
@@ -2476,7 +2598,7 @@
           </dLbls>
           <cat>
             <numRef>
-              <f>'Doughnut'!$B$10:$B$14</f>
+              <f>'Doughnut'!$A$10:$A$14</f>
             </numRef>
           </cat>
           <val>
@@ -2504,8 +2626,8 @@
           <yMode val="edge"/>
           <wMode val="factor"/>
           <hMode val="factor"/>
-          <x val="0.5600000000000001"/>
-          <y val="0.27"/>
+          <x val="0.74"/>
+          <y val="0.36"/>
           <w val="0.24"/>
           <h val="0.4"/>
         </manualLayout>
@@ -2515,7 +2637,7 @@
         <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
         <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
-            <a:defRPr sz="1400" b="0">
+            <a:defRPr sz="1500" b="0">
               <a:solidFill>
                 <a:srgbClr val="183958"/>
               </a:solidFill>
@@ -2525,7 +2647,7 @@
           <a:r>
             <a:t/>
           </a:r>
-          <a:endParaRPr sz="1400" b="0">
+          <a:endParaRPr sz="1500" b="0">
             <a:solidFill>
               <a:srgbClr val="183958"/>
             </a:solidFill>
@@ -3008,12 +3130,12 @@
 <c:userShapes xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing">
   <cdr:relSizeAnchor>
     <cdr:from>
-      <cdr:x>0.56</cdr:x>
-      <cdr:y>0.2</cdr:y>
+      <cdr:x>0.748</cdr:x>
+      <cdr:y>0.27</cdr:y>
     </cdr:from>
     <cdr:to>
-      <cdr:x>0.76</cdr:x>
-      <cdr:y>0.27</cdr:y>
+      <cdr:x>0.948</cdr:x>
+      <cdr:y>0.34</cdr:y>
     </cdr:to>
     <cdr:sp macro="" textlink="">
       <cdr:nvSpPr>
@@ -3911,29 +4033,29 @@
     <row r="7">
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Communications sent by channel</t>
+          <t>Communications by channel</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="C8" s="8">
-        <f>"  "&amp;C9&amp;"     "</f>
+        <f>" "&amp;C9&amp;"  "</f>
         <v/>
       </c>
       <c r="D8" s="8">
-        <f>"  "&amp;D9&amp;"     "</f>
+        <f>" "&amp;D9&amp;"  "</f>
         <v/>
       </c>
       <c r="E8" s="8">
-        <f>"  "&amp;E9&amp;"     "</f>
+        <f>" "&amp;E9&amp;"  "</f>
         <v/>
       </c>
       <c r="F8" s="8">
-        <f>"  "&amp;F9&amp;"     "</f>
+        <f>" "&amp;F9&amp;"  "</f>
         <v/>
       </c>
       <c r="G8" s="8">
-        <f>"  "&amp;G9&amp;"     "</f>
+        <f>" "&amp;G9&amp;"  "</f>
         <v/>
       </c>
     </row>
@@ -4159,25 +4281,25 @@
     <row r="7">
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Communications sent by channel</t>
+          <t>Communications by channel</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="C8" s="8">
-        <f>"  "&amp;C9&amp;"     "</f>
+        <f>" "&amp;C9&amp;"  "</f>
         <v/>
       </c>
       <c r="D8" s="8">
-        <f>"  "&amp;D9&amp;"     "</f>
+        <f>" "&amp;D9&amp;"  "</f>
         <v/>
       </c>
       <c r="E8" s="8">
-        <f>"  "&amp;E9&amp;"     "</f>
+        <f>" "&amp;E9&amp;"  "</f>
         <v/>
       </c>
       <c r="F8" s="8">
-        <f>"  "&amp;F9&amp;"     "</f>
+        <f>" "&amp;F9&amp;"  "</f>
         <v/>
       </c>
     </row>
@@ -4570,19 +4692,19 @@
     </row>
     <row r="8">
       <c r="C8" s="8">
-        <f>"  "&amp;C9&amp;"     "</f>
+        <f>" "&amp;C9&amp;"   "</f>
         <v/>
       </c>
       <c r="D8" s="8">
-        <f>"  "&amp;D9&amp;"     "</f>
+        <f>" "&amp;D9&amp;"   "</f>
         <v/>
       </c>
       <c r="E8" s="8">
-        <f>"  "&amp;E9&amp;"     "</f>
+        <f>" "&amp;E9&amp;"   "</f>
         <v/>
       </c>
       <c r="F8" s="8">
-        <f>"  "&amp;F9&amp;"     "</f>
+        <f>" "&amp;F9&amp;"   "</f>
         <v/>
       </c>
     </row>
@@ -4797,11 +4919,11 @@
     </row>
     <row r="8">
       <c r="C8" s="8">
-        <f>"  "&amp;C9&amp;"     "</f>
+        <f>" "&amp;C9&amp;"   "</f>
         <v/>
       </c>
       <c r="D8" s="8">
-        <f>"  "&amp;D9&amp;"     "</f>
+        <f>" "&amp;D9&amp;"   "</f>
         <v/>
       </c>
     </row>
@@ -5086,11 +5208,11 @@
     </row>
     <row r="8">
       <c r="C8" s="8">
-        <f>"  "&amp;C9&amp;"     "</f>
+        <f>" "&amp;C9&amp;"   "</f>
         <v/>
       </c>
       <c r="D8" s="8">
-        <f>"  "&amp;D9&amp;"     "</f>
+        <f>" "&amp;D9&amp;"   "</f>
         <v/>
       </c>
     </row>
@@ -5337,6 +5459,10 @@
       </c>
     </row>
     <row r="10">
+      <c r="A10" s="8">
+        <f>" "&amp;B10</f>
+        <v/>
+      </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
           <t>Web portal</t>
@@ -5347,6 +5473,10 @@
       </c>
     </row>
     <row r="11">
+      <c r="A11" s="8">
+        <f>" "&amp;B11</f>
+        <v/>
+      </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
           <t>Mobile app</t>
@@ -5357,6 +5487,10 @@
       </c>
     </row>
     <row r="12">
+      <c r="A12" s="8">
+        <f>" "&amp;B12</f>
+        <v/>
+      </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
           <t>Agent-assisted</t>
@@ -5367,6 +5501,10 @@
       </c>
     </row>
     <row r="13">
+      <c r="A13" s="8">
+        <f>" "&amp;B13</f>
+        <v/>
+      </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
           <t>Email link</t>
@@ -5377,6 +5515,10 @@
       </c>
     </row>
     <row r="14">
+      <c r="A14" s="8">
+        <f>" "&amp;B14</f>
+        <v/>
+      </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
           <t>Paper form</t>

</xml_diff>

<commit_message>
Excel: budget planning and program scoping workbooks; Segoe UI as the default font
Two new planning workbooks in the chart templates' look, with invented example content:
a functional budget plan (roll-up summary, adjustments, headcount, chart; plan year set
once) and a program scoping workbook (function inventories with effort, cost, readiness,
risk and timing; summary, decisions, dependencies, lists and definitions). The Templates
row becomes 'Excel Templates' with chart templates and planning workbooks.

All three workbooks now default to Segoe UI 10 for unstyled cells instead of Calibri 11.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/site/assets/downloads/SmartCommunications_Excel_Chart_Templates.xlsx
+++ b/site/assets/downloads/SmartCommunications_Excel_Chart_Templates.xlsx
@@ -33,10 +33,10 @@
   </numFmts>
   <fonts count="11">
     <font>
-      <name val="Calibri"/>
+      <name val="Segoe UI"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
+      <color rgb="00183958"/>
+      <sz val="10"/>
       <scheme val="minor"/>
     </font>
     <font>

</xml_diff>

<commit_message>
Excel templates: shaded formulas, darker input text, 11 pt type
Inputs are now Industry Blue text on white and calculated cells navy text on light blue,
as in the customers' own workbooks. Cell text steps up one size (body 11 pt) with an
18 pt default row height. The scoping summary's headline numbers are regular weight and
sit closer to their labels. Previews and the Excel row's wording updated to match.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/site/assets/downloads/SmartCommunications_Excel_Chart_Templates.xlsx
+++ b/site/assets/downloads/SmartCommunications_Excel_Chart_Templates.xlsx
@@ -36,13 +36,13 @@
       <name val="Segoe UI"/>
       <family val="2"/>
       <color rgb="00183958"/>
-      <sz val="10"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
       <name val="Segoe UI"/>
       <color rgb="00183958"/>
-      <sz val="10"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Segoe UI"/>
@@ -54,29 +54,29 @@
       <name val="Segoe UI"/>
       <b val="1"/>
       <color rgb="000E2030"/>
-      <sz val="12"/>
+      <sz val="13"/>
     </font>
     <font>
       <name val="Segoe UI"/>
-      <color rgb="000062A8"/>
+      <color rgb="000A3184"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <color rgb="00677C91"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Segoe UI"/>
-      <color rgb="00677C91"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="000062A8"/>
-      <sz val="11"/>
+      <color rgb="000A3184"/>
+      <sz val="12"/>
     </font>
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="10"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Segoe UI"/>
@@ -87,13 +87,13 @@
       <name val="Segoe UI"/>
       <b val="1"/>
       <color rgb="00183958"/>
-      <sz val="10"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
       <color rgb="00183958"/>
-      <sz val="11"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="12">
@@ -154,7 +154,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -167,6 +167,15 @@
         <color rgb="00D0DEEC"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00D0DEEC"/>
+      </bottom>
+      <diagonal/>
+    </border>
     <border/>
     <border>
       <bottom style="thick">
@@ -177,7 +186,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -185,9 +194,11 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -195,38 +206,37 @@
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" indent="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" indent="1"/>
     </xf>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" indent="1"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
+    <xf numFmtId="166" fontId="9" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="3" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="9" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="10" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="5" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="9" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="0" fillId="5" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -2681,7 +2691,7 @@
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="18230850" cy="609600"/>
+    <ext cx="20707350" cy="609600"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -2711,7 +2721,7 @@
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="20240625" cy="609600"/>
+    <ext cx="23002875" cy="609600"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -2763,7 +2773,7 @@
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="17954625" cy="609600"/>
+    <ext cx="20393025" cy="609600"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>
@@ -2815,7 +2825,7 @@
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="17954625" cy="609600"/>
+    <ext cx="20393025" cy="609600"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>
@@ -2867,7 +2877,7 @@
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="17954625" cy="609600"/>
+    <ext cx="20393025" cy="609600"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>
@@ -2919,7 +2929,7 @@
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="17954625" cy="609600"/>
+    <ext cx="20393025" cy="609600"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>
@@ -2971,7 +2981,7 @@
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="17954625" cy="609600"/>
+    <ext cx="20393025" cy="609600"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>
@@ -3023,7 +3033,7 @@
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="18373725" cy="609600"/>
+    <ext cx="20869275" cy="609600"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>
@@ -3075,7 +3085,7 @@
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="17954625" cy="609600"/>
+    <ext cx="20393025" cy="609600"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>
@@ -3105,7 +3115,7 @@
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="19069050" cy="609600"/>
+    <ext cx="21659850" cy="609600"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -3463,7 +3473,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:S21"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="18"/>
   <cols>
     <col width="2.5" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
@@ -3539,7 +3549,7 @@
     <row r="6">
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>2. Replace the sample data in the light-blue cells (dark blue text). Charts and formulas update automatically.</t>
+          <t>2. Replace the sample data: the values in blue text. Charts and formulas update automatically.</t>
         </is>
       </c>
     </row>
@@ -3570,7 +3580,7 @@
     <row r="11">
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Light-blue cell, dark blue text = edit me · plain cell, navy text = formula or label, leave it</t>
+          <t>Blue text on white = edit me · navy text on light blue = formula, leave it</t>
         </is>
       </c>
     </row>
@@ -3626,6 +3636,11 @@
       <c r="B21" s="5" t="inlineStr">
         <is>
           <t>Example input cell</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>Example calculated cell</t>
         </is>
       </c>
     </row>
@@ -3645,7 +3660,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:S20"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="18"/>
   <cols>
     <col width="2.5" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
@@ -3712,188 +3727,188 @@
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="25" t="inlineStr">
+      <c r="B7" s="26" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="C7" s="25" t="inlineStr">
+      <c r="C7" s="26" t="inlineStr">
         <is>
           <t>Color</t>
         </is>
       </c>
-      <c r="D7" s="25" t="inlineStr">
+      <c r="D7" s="26" t="inlineStr">
         <is>
           <t>HEX</t>
         </is>
       </c>
-      <c r="E7" s="25" t="inlineStr">
+      <c r="E7" s="26" t="inlineStr">
         <is>
           <t>Swatch</t>
         </is>
       </c>
-      <c r="F7" s="25" t="inlineStr">
+      <c r="F7" s="26" t="inlineStr">
         <is>
           <t>Use for</t>
         </is>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="B8" s="26" t="inlineStr">
+      <c r="B8" s="27" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="C8" s="26" t="inlineStr">
+      <c r="C8" s="27" t="inlineStr">
         <is>
           <t>Dodger</t>
         </is>
       </c>
-      <c r="D8" s="26" t="inlineStr">
+      <c r="D8" s="27" t="inlineStr">
         <is>
           <t>#0094FF</t>
         </is>
       </c>
-      <c r="E8" s="27" t="inlineStr"/>
-      <c r="F8" s="26" t="inlineStr">
+      <c r="E8" s="28" t="inlineStr"/>
+      <c r="F8" s="27" t="inlineStr">
         <is>
           <t>Lead series. Single-series charts use only this</t>
         </is>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="B9" s="26" t="inlineStr">
+      <c r="B9" s="27" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="C9" s="26" t="inlineStr">
+      <c r="C9" s="27" t="inlineStr">
         <is>
           <t>Indigo Dark</t>
         </is>
       </c>
-      <c r="D9" s="26" t="inlineStr">
+      <c r="D9" s="27" t="inlineStr">
         <is>
           <t>#661DEE</t>
         </is>
       </c>
-      <c r="E9" s="28" t="inlineStr"/>
-      <c r="F9" s="26" t="inlineStr">
+      <c r="E9" s="29" t="inlineStr"/>
+      <c r="F9" s="27" t="inlineStr">
         <is>
           <t>Second series, targets and comparisons</t>
         </is>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="B10" s="26" t="inlineStr">
+      <c r="B10" s="27" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="C10" s="26" t="inlineStr">
+      <c r="C10" s="27" t="inlineStr">
         <is>
           <t>Dodger Light</t>
         </is>
       </c>
-      <c r="D10" s="26" t="inlineStr">
+      <c r="D10" s="27" t="inlineStr">
         <is>
           <t>#57B8FF</t>
         </is>
       </c>
-      <c r="E10" s="29" t="inlineStr"/>
-      <c r="F10" s="26" t="inlineStr">
+      <c r="E10" s="30" t="inlineStr"/>
+      <c r="F10" s="27" t="inlineStr">
         <is>
           <t>Third series</t>
         </is>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="B11" s="26" t="inlineStr">
+      <c r="B11" s="27" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="C11" s="26" t="inlineStr">
+      <c r="C11" s="27" t="inlineStr">
         <is>
           <t>UI Blue Dark</t>
         </is>
       </c>
-      <c r="D11" s="26" t="inlineStr">
+      <c r="D11" s="27" t="inlineStr">
         <is>
           <t>#1344C1</t>
         </is>
       </c>
-      <c r="E11" s="30" t="inlineStr"/>
-      <c r="F11" s="26" t="inlineStr">
+      <c r="E11" s="31" t="inlineStr"/>
+      <c r="F11" s="27" t="inlineStr">
         <is>
           <t>Fourth series</t>
         </is>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="B12" s="26" t="inlineStr">
+      <c r="B12" s="27" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="C12" s="26" t="inlineStr">
+      <c r="C12" s="27" t="inlineStr">
         <is>
           <t>Indigo Light</t>
         </is>
       </c>
-      <c r="D12" s="26" t="inlineStr">
+      <c r="D12" s="27" t="inlineStr">
         <is>
           <t>#BE9DFA</t>
         </is>
       </c>
-      <c r="E12" s="31" t="inlineStr"/>
-      <c r="F12" s="26" t="inlineStr">
+      <c r="E12" s="32" t="inlineStr"/>
+      <c r="F12" s="27" t="inlineStr">
         <is>
           <t>Fifth series</t>
         </is>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="B13" s="26" t="inlineStr">
+      <c r="B13" s="27" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="C13" s="26" t="inlineStr">
+      <c r="C13" s="27" t="inlineStr">
         <is>
           <t>Dodger Dark</t>
         </is>
       </c>
-      <c r="D13" s="26" t="inlineStr">
+      <c r="D13" s="27" t="inlineStr">
         <is>
           <t>#0062A8</t>
         </is>
       </c>
-      <c r="E13" s="32" t="inlineStr"/>
-      <c r="F13" s="26" t="inlineStr">
+      <c r="E13" s="33" t="inlineStr"/>
+      <c r="F13" s="27" t="inlineStr">
         <is>
           <t>Sixth series, or fold the rest into 'Other'</t>
         </is>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="B14" s="26" t="inlineStr">
+      <c r="B14" s="27" t="inlineStr">
         <is>
           <t>Dark</t>
         </is>
       </c>
-      <c r="C14" s="26" t="inlineStr">
+      <c r="C14" s="27" t="inlineStr">
         <is>
           <t>On Tiber slides</t>
         </is>
       </c>
-      <c r="D14" s="26" t="inlineStr">
+      <c r="D14" s="27" t="inlineStr">
         <is>
           <t>#0094FF · #661DEE · #0062A8 · #9963FD</t>
         </is>
       </c>
-      <c r="E14" s="26" t="inlineStr"/>
-      <c r="F14" s="26" t="inlineStr">
+      <c r="E14" s="27" t="inlineStr"/>
+      <c r="F14" s="27" t="inlineStr">
         <is>
           <t>Four series at most on dark</t>
         </is>
@@ -3957,7 +3972,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:S14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="18"/>
   <cols>
     <col width="2.5" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
@@ -4019,168 +4034,172 @@
     <row r="4">
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Edit the light-blue cells: the chart updates automatically. Copy the chart into PowerPoint or Word.</t>
+          <t>Edit the blue values: the chart updates automatically. Copy the chart into PowerPoint or Word.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>Chart title</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>Communications by channel</t>
         </is>
       </c>
+      <c r="C7" s="9" t="n"/>
+      <c r="D7" s="9" t="n"/>
+      <c r="E7" s="9" t="n"/>
+      <c r="F7" s="9" t="n"/>
     </row>
     <row r="8">
-      <c r="C8" s="8">
+      <c r="C8" s="10">
         <f>" "&amp;C9&amp;"  "</f>
         <v/>
       </c>
-      <c r="D8" s="8">
+      <c r="D8" s="10">
         <f>" "&amp;D9&amp;"  "</f>
         <v/>
       </c>
-      <c r="E8" s="8">
+      <c r="E8" s="10">
         <f>" "&amp;E9&amp;"  "</f>
         <v/>
       </c>
-      <c r="F8" s="8">
+      <c r="F8" s="10">
         <f>" "&amp;F9&amp;"  "</f>
         <v/>
       </c>
-      <c r="G8" s="8">
+      <c r="G8" s="10">
         <f>" "&amp;G9&amp;"  "</f>
         <v/>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="11" t="inlineStr">
         <is>
           <t>Quarter</t>
         </is>
       </c>
-      <c r="C9" s="10" t="inlineStr">
+      <c r="C9" s="12" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="D9" s="10" t="inlineStr">
+      <c r="D9" s="12" t="inlineStr">
         <is>
           <t>Print</t>
         </is>
       </c>
-      <c r="E9" s="10" t="inlineStr">
+      <c r="E9" s="12" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="F9" s="10" t="inlineStr">
+      <c r="F9" s="12" t="inlineStr">
         <is>
           <t>Portal</t>
         </is>
       </c>
-      <c r="G9" s="10" t="inlineStr">
+      <c r="G9" s="12" t="inlineStr">
         <is>
           <t>App</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="11" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>Q1</t>
         </is>
       </c>
-      <c r="C10" s="12" t="n">
+      <c r="C10" s="13" t="n">
         <v>42000</v>
       </c>
-      <c r="D10" s="12" t="n">
+      <c r="D10" s="13" t="n">
         <v>31000</v>
       </c>
-      <c r="E10" s="12" t="n">
+      <c r="E10" s="13" t="n">
         <v>12000</v>
       </c>
-      <c r="F10" s="12" t="n">
+      <c r="F10" s="13" t="n">
         <v>21000</v>
       </c>
-      <c r="G10" s="12" t="n">
+      <c r="G10" s="13" t="n">
         <v>8000</v>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="11" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>Q2</t>
         </is>
       </c>
-      <c r="C11" s="12" t="n">
+      <c r="C11" s="13" t="n">
         <v>46500</v>
       </c>
-      <c r="D11" s="12" t="n">
+      <c r="D11" s="13" t="n">
         <v>29800</v>
       </c>
-      <c r="E11" s="12" t="n">
+      <c r="E11" s="13" t="n">
         <v>15400</v>
       </c>
-      <c r="F11" s="12" t="n">
+      <c r="F11" s="13" t="n">
         <v>24000</v>
       </c>
-      <c r="G11" s="12" t="n">
+      <c r="G11" s="13" t="n">
         <v>11500</v>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="11" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>Q3</t>
         </is>
       </c>
-      <c r="C12" s="12" t="n">
+      <c r="C12" s="13" t="n">
         <v>51200</v>
       </c>
-      <c r="D12" s="12" t="n">
+      <c r="D12" s="13" t="n">
         <v>27600</v>
       </c>
-      <c r="E12" s="12" t="n">
+      <c r="E12" s="13" t="n">
         <v>18900</v>
       </c>
-      <c r="F12" s="12" t="n">
+      <c r="F12" s="13" t="n">
         <v>26500</v>
       </c>
-      <c r="G12" s="12" t="n">
+      <c r="G12" s="13" t="n">
         <v>15800</v>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="11" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>Q4</t>
         </is>
       </c>
-      <c r="C13" s="12" t="n">
+      <c r="C13" s="13" t="n">
         <v>55800</v>
       </c>
-      <c r="D13" s="12" t="n">
+      <c r="D13" s="13" t="n">
         <v>26100</v>
       </c>
-      <c r="E13" s="12" t="n">
+      <c r="E13" s="13" t="n">
         <v>22300</v>
       </c>
-      <c r="F13" s="12" t="n">
+      <c r="F13" s="13" t="n">
         <v>29900</v>
       </c>
-      <c r="G13" s="12" t="n">
+      <c r="G13" s="13" t="n">
         <v>19400</v>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="6" t="inlineStr">
+      <c r="B14" s="7" t="inlineStr">
         <is>
           <t>Sample data is illustrative. Replace it with your own and cite the source under the table.</t>
         </is>
@@ -4205,7 +4224,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:S14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="18"/>
   <cols>
     <col width="2.5" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
@@ -4267,147 +4286,151 @@
     <row r="4">
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Edit the light-blue cells: the chart updates automatically. Copy the chart into PowerPoint or Word. This version is styled for Tiber (dark) slides.</t>
+          <t>Edit the blue values: the chart updates automatically. Copy the chart into PowerPoint or Word. This version is styled for Tiber (dark) slides.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>Chart title</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>Communications by channel</t>
         </is>
       </c>
+      <c r="C7" s="9" t="n"/>
+      <c r="D7" s="9" t="n"/>
+      <c r="E7" s="9" t="n"/>
+      <c r="F7" s="9" t="n"/>
     </row>
     <row r="8">
-      <c r="C8" s="8">
+      <c r="C8" s="10">
         <f>" "&amp;C9&amp;"  "</f>
         <v/>
       </c>
-      <c r="D8" s="8">
+      <c r="D8" s="10">
         <f>" "&amp;D9&amp;"  "</f>
         <v/>
       </c>
-      <c r="E8" s="8">
+      <c r="E8" s="10">
         <f>" "&amp;E9&amp;"  "</f>
         <v/>
       </c>
-      <c r="F8" s="8">
+      <c r="F8" s="10">
         <f>" "&amp;F9&amp;"  "</f>
         <v/>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="11" t="inlineStr">
         <is>
           <t>Quarter</t>
         </is>
       </c>
-      <c r="C9" s="10" t="inlineStr">
+      <c r="C9" s="12" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="D9" s="10" t="inlineStr">
+      <c r="D9" s="12" t="inlineStr">
         <is>
           <t>Print</t>
         </is>
       </c>
-      <c r="E9" s="10" t="inlineStr">
+      <c r="E9" s="12" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="F9" s="10" t="inlineStr">
+      <c r="F9" s="12" t="inlineStr">
         <is>
           <t>Portal</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="11" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>Q1</t>
         </is>
       </c>
-      <c r="C10" s="12" t="n">
+      <c r="C10" s="13" t="n">
         <v>42000</v>
       </c>
-      <c r="D10" s="12" t="n">
+      <c r="D10" s="13" t="n">
         <v>31000</v>
       </c>
-      <c r="E10" s="12" t="n">
+      <c r="E10" s="13" t="n">
         <v>12000</v>
       </c>
-      <c r="F10" s="12" t="n">
+      <c r="F10" s="13" t="n">
         <v>21000</v>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="11" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>Q2</t>
         </is>
       </c>
-      <c r="C11" s="12" t="n">
+      <c r="C11" s="13" t="n">
         <v>46500</v>
       </c>
-      <c r="D11" s="12" t="n">
+      <c r="D11" s="13" t="n">
         <v>29800</v>
       </c>
-      <c r="E11" s="12" t="n">
+      <c r="E11" s="13" t="n">
         <v>15400</v>
       </c>
-      <c r="F11" s="12" t="n">
+      <c r="F11" s="13" t="n">
         <v>24000</v>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="11" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>Q3</t>
         </is>
       </c>
-      <c r="C12" s="12" t="n">
+      <c r="C12" s="13" t="n">
         <v>51200</v>
       </c>
-      <c r="D12" s="12" t="n">
+      <c r="D12" s="13" t="n">
         <v>27600</v>
       </c>
-      <c r="E12" s="12" t="n">
+      <c r="E12" s="13" t="n">
         <v>18900</v>
       </c>
-      <c r="F12" s="12" t="n">
+      <c r="F12" s="13" t="n">
         <v>26500</v>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="11" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>Q4</t>
         </is>
       </c>
-      <c r="C13" s="12" t="n">
+      <c r="C13" s="13" t="n">
         <v>55800</v>
       </c>
-      <c r="D13" s="12" t="n">
+      <c r="D13" s="13" t="n">
         <v>26100</v>
       </c>
-      <c r="E13" s="12" t="n">
+      <c r="E13" s="13" t="n">
         <v>22300</v>
       </c>
-      <c r="F13" s="12" t="n">
+      <c r="F13" s="13" t="n">
         <v>29900</v>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="6" t="inlineStr">
+      <c r="B14" s="7" t="inlineStr">
         <is>
           <t>Sample data is illustrative. Replace it with your own and cite the source under the table.</t>
         </is>
@@ -4432,7 +4455,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:S16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="18"/>
   <cols>
     <col width="2.5" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
@@ -4499,93 +4522,97 @@
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>Chart title</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>Templates migrated by business unit</t>
         </is>
       </c>
+      <c r="C7" s="9" t="n"/>
+      <c r="D7" s="9" t="n"/>
+      <c r="E7" s="9" t="n"/>
+      <c r="F7" s="9" t="n"/>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="11" t="inlineStr">
         <is>
           <t>Business unit</t>
         </is>
       </c>
-      <c r="C9" s="10" t="inlineStr">
+      <c r="C9" s="12" t="inlineStr">
         <is>
           <t>Templates</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="11" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>Claims</t>
         </is>
       </c>
-      <c r="C10" s="12" t="n">
+      <c r="C10" s="13" t="n">
         <v>412</v>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="11" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>Policy servicing</t>
         </is>
       </c>
-      <c r="C11" s="12" t="n">
+      <c r="C11" s="13" t="n">
         <v>356</v>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="11" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>Billing</t>
         </is>
       </c>
-      <c r="C12" s="12" t="n">
+      <c r="C12" s="13" t="n">
         <v>298</v>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="11" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>Onboarding</t>
         </is>
       </c>
-      <c r="C13" s="12" t="n">
+      <c r="C13" s="13" t="n">
         <v>241</v>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="11" t="inlineStr">
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>Complaints</t>
         </is>
       </c>
-      <c r="C14" s="12" t="n">
+      <c r="C14" s="13" t="n">
         <v>167</v>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="11" t="inlineStr">
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>Marketing</t>
         </is>
       </c>
-      <c r="C15" s="12" t="n">
+      <c r="C15" s="13" t="n">
         <v>102</v>
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="6" t="inlineStr">
+      <c r="B16" s="7" t="inlineStr">
         <is>
           <t>Sample data is illustrative. Replace it with your own and cite the source under the table.</t>
         </is>
@@ -4610,7 +4637,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:S14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="18"/>
   <cols>
     <col width="2.5" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
@@ -4677,142 +4704,146 @@
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>Chart title</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>Channel mix by quarter</t>
         </is>
       </c>
+      <c r="C7" s="9" t="n"/>
+      <c r="D7" s="9" t="n"/>
+      <c r="E7" s="9" t="n"/>
+      <c r="F7" s="9" t="n"/>
     </row>
     <row r="8">
-      <c r="C8" s="8">
+      <c r="C8" s="10">
         <f>" "&amp;C9&amp;"   "</f>
         <v/>
       </c>
-      <c r="D8" s="8">
+      <c r="D8" s="10">
         <f>" "&amp;D9&amp;"   "</f>
         <v/>
       </c>
-      <c r="E8" s="8">
+      <c r="E8" s="10">
         <f>" "&amp;E9&amp;"   "</f>
         <v/>
       </c>
-      <c r="F8" s="8">
+      <c r="F8" s="10">
         <f>" "&amp;F9&amp;"   "</f>
         <v/>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="11" t="inlineStr">
         <is>
           <t>Quarter</t>
         </is>
       </c>
-      <c r="C9" s="10" t="inlineStr">
+      <c r="C9" s="12" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="D9" s="10" t="inlineStr">
+      <c r="D9" s="12" t="inlineStr">
         <is>
           <t>Portal</t>
         </is>
       </c>
-      <c r="E9" s="10" t="inlineStr">
+      <c r="E9" s="12" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="F9" s="10" t="inlineStr">
+      <c r="F9" s="12" t="inlineStr">
         <is>
           <t>Print</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="11" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>Q1</t>
         </is>
       </c>
-      <c r="C10" s="13" t="n">
+      <c r="C10" s="14" t="n">
         <v>38</v>
       </c>
-      <c r="D10" s="13" t="n">
+      <c r="D10" s="14" t="n">
         <v>14</v>
       </c>
-      <c r="E10" s="13" t="n">
+      <c r="E10" s="14" t="n">
         <v>11</v>
       </c>
-      <c r="F10" s="13" t="n">
+      <c r="F10" s="14" t="n">
         <v>37</v>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="11" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>Q2</t>
         </is>
       </c>
-      <c r="C11" s="13" t="n">
+      <c r="C11" s="14" t="n">
         <v>41</v>
       </c>
-      <c r="D11" s="13" t="n">
+      <c r="D11" s="14" t="n">
         <v>17</v>
       </c>
-      <c r="E11" s="13" t="n">
+      <c r="E11" s="14" t="n">
         <v>13</v>
       </c>
-      <c r="F11" s="13" t="n">
+      <c r="F11" s="14" t="n">
         <v>29</v>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="11" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>Q3</t>
         </is>
       </c>
-      <c r="C12" s="13" t="n">
+      <c r="C12" s="14" t="n">
         <v>44</v>
       </c>
-      <c r="D12" s="13" t="n">
+      <c r="D12" s="14" t="n">
         <v>19</v>
       </c>
-      <c r="E12" s="13" t="n">
+      <c r="E12" s="14" t="n">
         <v>14</v>
       </c>
-      <c r="F12" s="13" t="n">
+      <c r="F12" s="14" t="n">
         <v>23</v>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="11" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>Q4</t>
         </is>
       </c>
-      <c r="C13" s="13" t="n">
+      <c r="C13" s="14" t="n">
         <v>46</v>
       </c>
-      <c r="D13" s="13" t="n">
+      <c r="D13" s="14" t="n">
         <v>22</v>
       </c>
-      <c r="E13" s="13" t="n">
+      <c r="E13" s="14" t="n">
         <v>16</v>
       </c>
-      <c r="F13" s="13" t="n">
+      <c r="F13" s="14" t="n">
         <v>16</v>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="6" t="inlineStr">
+      <c r="B14" s="7" t="inlineStr">
         <is>
           <t>Sample data is illustrative. Replace it with your own and cite the source under the table. Values are percent of volume and add up to 100.</t>
         </is>
@@ -4837,7 +4868,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:S22"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="18"/>
   <cols>
     <col width="2.5" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
@@ -4904,204 +4935,208 @@
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>Chart title</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>Average days to update a template</t>
         </is>
       </c>
+      <c r="C7" s="9" t="n"/>
+      <c r="D7" s="9" t="n"/>
+      <c r="E7" s="9" t="n"/>
+      <c r="F7" s="9" t="n"/>
     </row>
     <row r="8">
-      <c r="C8" s="8">
+      <c r="C8" s="10">
         <f>" "&amp;C9&amp;"   "</f>
         <v/>
       </c>
-      <c r="D8" s="8">
+      <c r="D8" s="10">
         <f>" "&amp;D9&amp;"   "</f>
         <v/>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="11" t="inlineStr">
         <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="C9" s="10" t="inlineStr">
+      <c r="C9" s="12" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="D9" s="10" t="inlineStr">
+      <c r="D9" s="12" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="11" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>Jan</t>
         </is>
       </c>
-      <c r="C10" s="12" t="n">
+      <c r="C10" s="13" t="n">
         <v>21</v>
       </c>
-      <c r="D10" s="12" t="n">
+      <c r="D10" s="13" t="n">
         <v>24</v>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="11" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>Feb</t>
         </is>
       </c>
-      <c r="C11" s="12" t="n">
+      <c r="C11" s="13" t="n">
         <v>19</v>
       </c>
-      <c r="D11" s="12" t="n">
+      <c r="D11" s="13" t="n">
         <v>24</v>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="11" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>Mar</t>
         </is>
       </c>
-      <c r="C12" s="12" t="n">
+      <c r="C12" s="13" t="n">
         <v>18</v>
       </c>
-      <c r="D12" s="12" t="n">
+      <c r="D12" s="13" t="n">
         <v>23</v>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="11" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>Apr</t>
         </is>
       </c>
-      <c r="C13" s="12" t="n">
+      <c r="C13" s="13" t="n">
         <v>16</v>
       </c>
-      <c r="D13" s="12" t="n">
+      <c r="D13" s="13" t="n">
         <v>23</v>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="11" t="inlineStr">
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>May</t>
         </is>
       </c>
-      <c r="C14" s="12" t="n">
+      <c r="C14" s="13" t="n">
         <v>15</v>
       </c>
-      <c r="D14" s="12" t="n">
+      <c r="D14" s="13" t="n">
         <v>22</v>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="11" t="inlineStr">
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>Jun</t>
         </is>
       </c>
-      <c r="C15" s="12" t="n">
+      <c r="C15" s="13" t="n">
         <v>13</v>
       </c>
-      <c r="D15" s="12" t="n">
+      <c r="D15" s="13" t="n">
         <v>22</v>
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="11" t="inlineStr">
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>Jul</t>
         </is>
       </c>
-      <c r="C16" s="12" t="n">
+      <c r="C16" s="13" t="n">
         <v>12</v>
       </c>
-      <c r="D16" s="12" t="n">
+      <c r="D16" s="13" t="n">
         <v>21</v>
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="11" t="inlineStr">
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>Aug</t>
         </is>
       </c>
-      <c r="C17" s="12" t="n">
+      <c r="C17" s="13" t="n">
         <v>11</v>
       </c>
-      <c r="D17" s="12" t="n">
+      <c r="D17" s="13" t="n">
         <v>21</v>
       </c>
     </row>
     <row r="18">
-      <c r="B18" s="11" t="inlineStr">
+      <c r="B18" s="5" t="inlineStr">
         <is>
           <t>Sep</t>
         </is>
       </c>
-      <c r="C18" s="12" t="n">
+      <c r="C18" s="13" t="n">
         <v>10</v>
       </c>
-      <c r="D18" s="12" t="n">
+      <c r="D18" s="13" t="n">
         <v>21</v>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="11" t="inlineStr">
+      <c r="B19" s="5" t="inlineStr">
         <is>
           <t>Oct</t>
         </is>
       </c>
-      <c r="C19" s="12" t="n">
+      <c r="C19" s="13" t="n">
         <v>9</v>
       </c>
-      <c r="D19" s="12" t="n">
+      <c r="D19" s="13" t="n">
         <v>20</v>
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="11" t="inlineStr">
+      <c r="B20" s="5" t="inlineStr">
         <is>
           <t>Nov</t>
         </is>
       </c>
-      <c r="C20" s="12" t="n">
+      <c r="C20" s="13" t="n">
         <v>8</v>
       </c>
-      <c r="D20" s="12" t="n">
+      <c r="D20" s="13" t="n">
         <v>20</v>
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="11" t="inlineStr">
+      <c r="B21" s="5" t="inlineStr">
         <is>
           <t>Dec</t>
         </is>
       </c>
-      <c r="C21" s="12" t="n">
+      <c r="C21" s="13" t="n">
         <v>7</v>
       </c>
-      <c r="D21" s="12" t="n">
+      <c r="D21" s="13" t="n">
         <v>20</v>
       </c>
     </row>
     <row r="22">
-      <c r="B22" s="6" t="inlineStr">
+      <c r="B22" s="7" t="inlineStr">
         <is>
           <t>Sample data is illustrative. Replace it with your own and cite the source under the table.</t>
         </is>
@@ -5126,7 +5161,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:S16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="18"/>
   <cols>
     <col width="2.5" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
@@ -5193,155 +5228,159 @@
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>Chart title</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>Templates migrated vs. target</t>
         </is>
       </c>
+      <c r="C7" s="9" t="n"/>
+      <c r="D7" s="9" t="n"/>
+      <c r="E7" s="9" t="n"/>
+      <c r="F7" s="9" t="n"/>
     </row>
     <row r="8">
-      <c r="C8" s="8">
+      <c r="C8" s="10">
         <f>" "&amp;C9&amp;"   "</f>
         <v/>
       </c>
-      <c r="D8" s="8">
+      <c r="D8" s="10">
         <f>" "&amp;D9&amp;"   "</f>
         <v/>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="11" t="inlineStr">
         <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="C9" s="10" t="inlineStr">
+      <c r="C9" s="12" t="inlineStr">
         <is>
           <t>Migrated</t>
         </is>
       </c>
-      <c r="D9" s="10" t="inlineStr">
+      <c r="D9" s="12" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="E9" s="10" t="inlineStr">
+      <c r="E9" s="12" t="inlineStr">
         <is>
           <t>vs. target</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="11" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>Jan</t>
         </is>
       </c>
-      <c r="C10" s="12" t="n">
+      <c r="C10" s="13" t="n">
         <v>182</v>
       </c>
-      <c r="D10" s="12" t="n">
+      <c r="D10" s="13" t="n">
         <v>200</v>
       </c>
-      <c r="E10" s="14">
+      <c r="E10" s="15">
         <f>IF(D10=0,0,C10/D10-1)</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="11" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>Feb</t>
         </is>
       </c>
-      <c r="C11" s="12" t="n">
+      <c r="C11" s="13" t="n">
         <v>196</v>
       </c>
-      <c r="D11" s="12" t="n">
+      <c r="D11" s="13" t="n">
         <v>210</v>
       </c>
-      <c r="E11" s="14">
+      <c r="E11" s="15">
         <f>IF(D11=0,0,C11/D11-1)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="11" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>Mar</t>
         </is>
       </c>
-      <c r="C12" s="12" t="n">
+      <c r="C12" s="13" t="n">
         <v>228</v>
       </c>
-      <c r="D12" s="12" t="n">
+      <c r="D12" s="13" t="n">
         <v>220</v>
       </c>
-      <c r="E12" s="14">
+      <c r="E12" s="15">
         <f>IF(D12=0,0,C12/D12-1)</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="11" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>Apr</t>
         </is>
       </c>
-      <c r="C13" s="12" t="n">
+      <c r="C13" s="13" t="n">
         <v>241</v>
       </c>
-      <c r="D13" s="12" t="n">
+      <c r="D13" s="13" t="n">
         <v>235</v>
       </c>
-      <c r="E13" s="14">
+      <c r="E13" s="15">
         <f>IF(D13=0,0,C13/D13-1)</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="11" t="inlineStr">
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>May</t>
         </is>
       </c>
-      <c r="C14" s="12" t="n">
+      <c r="C14" s="13" t="n">
         <v>263</v>
       </c>
-      <c r="D14" s="12" t="n">
+      <c r="D14" s="13" t="n">
         <v>250</v>
       </c>
-      <c r="E14" s="14">
+      <c r="E14" s="15">
         <f>IF(D14=0,0,C14/D14-1)</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="11" t="inlineStr">
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>Jun</t>
         </is>
       </c>
-      <c r="C15" s="12" t="n">
+      <c r="C15" s="13" t="n">
         <v>288</v>
       </c>
-      <c r="D15" s="12" t="n">
+      <c r="D15" s="13" t="n">
         <v>265</v>
       </c>
-      <c r="E15" s="14">
+      <c r="E15" s="15">
         <f>IF(D15=0,0,C15/D15-1)</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="6" t="inlineStr">
+      <c r="B16" s="7" t="inlineStr">
         <is>
           <t>Sample data is illustrative. Replace it with your own and cite the source under the table.</t>
         </is>
@@ -5366,7 +5405,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:S16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="18"/>
   <cols>
     <col width="2.5" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
@@ -5433,114 +5472,118 @@
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>Chart title</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>Where customers start a form</t>
         </is>
       </c>
+      <c r="C7" s="9" t="n"/>
+      <c r="D7" s="9" t="n"/>
+      <c r="E7" s="9" t="n"/>
+      <c r="F7" s="9" t="n"/>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="11" t="inlineStr">
         <is>
           <t>Channel</t>
         </is>
       </c>
-      <c r="C9" s="10" t="inlineStr">
+      <c r="C9" s="12" t="inlineStr">
         <is>
           <t>Share</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="8">
+      <c r="A10" s="10">
         <f>" "&amp;B10</f>
         <v/>
       </c>
-      <c r="B10" s="11" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>Web portal</t>
         </is>
       </c>
-      <c r="C10" s="15" t="n">
+      <c r="C10" s="16" t="n">
         <v>0.38</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="8">
+      <c r="A11" s="10">
         <f>" "&amp;B11</f>
         <v/>
       </c>
-      <c r="B11" s="11" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>Mobile app</t>
         </is>
       </c>
-      <c r="C11" s="15" t="n">
+      <c r="C11" s="16" t="n">
         <v>0.24</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="8">
+      <c r="A12" s="10">
         <f>" "&amp;B12</f>
         <v/>
       </c>
-      <c r="B12" s="11" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>Agent-assisted</t>
         </is>
       </c>
-      <c r="C12" s="15" t="n">
+      <c r="C12" s="16" t="n">
         <v>0.17</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="8">
+      <c r="A13" s="10">
         <f>" "&amp;B13</f>
         <v/>
       </c>
-      <c r="B13" s="11" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>Email link</t>
         </is>
       </c>
-      <c r="C13" s="15" t="n">
+      <c r="C13" s="16" t="n">
         <v>0.13</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="8">
+      <c r="A14" s="10">
         <f>" "&amp;B14</f>
         <v/>
       </c>
-      <c r="B14" s="11" t="inlineStr">
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>Paper form</t>
         </is>
       </c>
-      <c r="C14" s="15" t="n">
+      <c r="C14" s="16" t="n">
         <v>0.08</v>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="16" t="inlineStr">
+      <c r="B15" s="17" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="C15" s="17">
+      <c r="C15" s="18">
         <f>SUM(C10:C14)</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="6" t="inlineStr">
+      <c r="B16" s="7" t="inlineStr">
         <is>
           <t>Sample data is illustrative. Replace it with your own and cite the source under the table. Shares should total 100%.</t>
         </is>
@@ -5565,7 +5608,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:S12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="18"/>
   <cols>
     <col width="2.5" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
@@ -5627,144 +5670,144 @@
     <row r="4">
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>A formatted table with in-cell bars, for when a chart is too much. Edit the light-blue cells.</t>
+          <t>A formatted table with in-cell bars, for when a chart is too much. Edit the blue values.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="B7" s="9" t="inlineStr">
+      <c r="B7" s="11" t="inlineStr">
         <is>
           <t>Program</t>
         </is>
       </c>
-      <c r="C7" s="10" t="inlineStr">
+      <c r="C7" s="12" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="D7" s="10" t="inlineStr">
+      <c r="D7" s="12" t="inlineStr">
         <is>
           <t>Actual</t>
         </is>
       </c>
-      <c r="E7" s="10" t="inlineStr">
+      <c r="E7" s="12" t="inlineStr">
         <is>
           <t>vs. target</t>
         </is>
       </c>
-      <c r="F7" s="10" t="inlineStr"/>
-      <c r="G7" s="9" t="inlineStr">
+      <c r="F7" s="12" t="inlineStr"/>
+      <c r="G7" s="11" t="inlineStr">
         <is>
           <t>Progress</t>
         </is>
       </c>
     </row>
     <row r="8" ht="24" customHeight="1">
-      <c r="B8" s="18" t="inlineStr">
+      <c r="B8" s="19" t="inlineStr">
         <is>
           <t>Template consolidation</t>
         </is>
       </c>
-      <c r="C8" s="19" t="n">
+      <c r="C8" s="20" t="n">
         <v>1200</v>
       </c>
-      <c r="D8" s="19" t="n">
+      <c r="D8" s="20" t="n">
         <v>1056</v>
       </c>
-      <c r="E8" s="20">
+      <c r="E8" s="21">
         <f>IF(C8=0,0,D8/C8-1)</f>
         <v/>
       </c>
-      <c r="F8" s="21" t="n"/>
-      <c r="G8" s="22">
+      <c r="F8" s="22" t="n"/>
+      <c r="G8" s="23">
         <f>IF(C8=0,0,MIN(1,D8/C8))</f>
         <v/>
       </c>
-      <c r="H8" s="23">
+      <c r="H8" s="24">
         <f>G8</f>
         <v/>
       </c>
     </row>
     <row r="9" ht="24" customHeight="1">
-      <c r="B9" s="18" t="inlineStr">
+      <c r="B9" s="19" t="inlineStr">
         <is>
           <t>Digital adoption</t>
         </is>
       </c>
-      <c r="C9" s="24" t="n">
+      <c r="C9" s="25" t="n">
         <v>0.6</v>
       </c>
-      <c r="D9" s="24" t="n">
+      <c r="D9" s="25" t="n">
         <v>0.54</v>
       </c>
-      <c r="E9" s="20">
+      <c r="E9" s="21">
         <f>IF(C9=0,0,D9/C9-1)</f>
         <v/>
       </c>
-      <c r="F9" s="21" t="n"/>
-      <c r="G9" s="22">
+      <c r="F9" s="22" t="n"/>
+      <c r="G9" s="23">
         <f>IF(C9=0,0,MIN(1,D9/C9))</f>
         <v/>
       </c>
-      <c r="H9" s="23">
+      <c r="H9" s="24">
         <f>G9</f>
         <v/>
       </c>
     </row>
     <row r="10" ht="24" customHeight="1">
-      <c r="B10" s="18" t="inlineStr">
+      <c r="B10" s="19" t="inlineStr">
         <is>
           <t>Straight-through processing</t>
         </is>
       </c>
-      <c r="C10" s="24" t="n">
+      <c r="C10" s="25" t="n">
         <v>0.85</v>
       </c>
-      <c r="D10" s="24" t="n">
+      <c r="D10" s="25" t="n">
         <v>0.8100000000000001</v>
       </c>
-      <c r="E10" s="20">
+      <c r="E10" s="21">
         <f>IF(C10=0,0,D10/C10-1)</f>
         <v/>
       </c>
-      <c r="F10" s="21" t="n"/>
-      <c r="G10" s="22">
+      <c r="F10" s="22" t="n"/>
+      <c r="G10" s="23">
         <f>IF(C10=0,0,MIN(1,D10/C10))</f>
         <v/>
       </c>
-      <c r="H10" s="23">
+      <c r="H10" s="24">
         <f>G10</f>
         <v/>
       </c>
     </row>
     <row r="11" ht="24" customHeight="1">
-      <c r="B11" s="18" t="inlineStr">
+      <c r="B11" s="19" t="inlineStr">
         <is>
           <t>Self-service forms live</t>
         </is>
       </c>
-      <c r="C11" s="19" t="n">
+      <c r="C11" s="20" t="n">
         <v>40</v>
       </c>
-      <c r="D11" s="19" t="n">
+      <c r="D11" s="20" t="n">
         <v>46</v>
       </c>
-      <c r="E11" s="20">
+      <c r="E11" s="21">
         <f>IF(C11=0,0,D11/C11-1)</f>
         <v/>
       </c>
-      <c r="F11" s="21" t="n"/>
-      <c r="G11" s="22">
+      <c r="F11" s="22" t="n"/>
+      <c r="G11" s="23">
         <f>IF(C11=0,0,MIN(1,D11/C11))</f>
         <v/>
       </c>
-      <c r="H11" s="23">
+      <c r="H11" s="24">
         <f>G11</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="6" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>Sample data is illustrative. Replace it with your own and cite the source under the table. 'vs. target' and 'Progress' are formulas; bars stop at 100%.</t>
         </is>

</xml_diff>